<commit_message>
Excel-Sheet zu finanzmathematischen Faktoren aktualisiert.
</commit_message>
<xml_diff>
--- a/Beispiele/Finanzmathematische_Faktoren.xlsx
+++ b/Beispiele/Finanzmathematische_Faktoren.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11011"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11020"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/stefan/Github/wirtschaftsmathematik/Beispiele/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FC69EEBA-8DA3-2A46-AD2A-C53A183E8A8A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0EA20AA6-30B9-8F42-9C66-907877206D5B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="34560" windowHeight="20620" xr2:uid="{1E627648-D751-2F4E-98FD-25D645E85C86}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
     <sheet name="Tabelle2" sheetId="2" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="181029"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -73,9 +73,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="2">
+  <numFmts count="4">
     <numFmt numFmtId="43" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
     <numFmt numFmtId="164" formatCode="_-* #,##0.000_-;\-* #,##0.000_-;_-* &quot;-&quot;??_-;_-@_-"/>
+    <numFmt numFmtId="165" formatCode="0.0%"/>
+    <numFmt numFmtId="166" formatCode="_-* #,##0.000\ _€_-;\-* #,##0.000\ _€_-;_-* &quot;-&quot;???\ _€_-;_-@_-"/>
   </numFmts>
   <fonts count="3" x14ac:knownFonts="1">
     <font>
@@ -284,7 +286,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -305,15 +307,6 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="9" fontId="2" fillId="3" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="2" fillId="3" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="2" fillId="3" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -324,6 +317,16 @@
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="165" fontId="2" fillId="3" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="2" fillId="3" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="2" fillId="3" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Komma" xfId="1" builtinId="3"/>
@@ -659,67 +662,68 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D132AD33-D6FE-B04D-BE81-942B50447162}">
-  <dimension ref="A1:M17"/>
+  <dimension ref="A1:M19"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="10.83203125" style="1"/>
+    <col min="2" max="2" width="13" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:13" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A1" s="3"/>
-      <c r="B1" s="12" t="s">
-        <v>2</v>
-      </c>
-      <c r="C1" s="12"/>
-      <c r="D1" s="12"/>
-      <c r="E1" s="12"/>
-      <c r="F1" s="12"/>
-      <c r="G1" s="12"/>
-      <c r="H1" s="12"/>
-      <c r="I1" s="12"/>
-      <c r="J1" s="12"/>
-      <c r="K1" s="12"/>
-      <c r="L1" s="12"/>
-      <c r="M1" s="13"/>
+      <c r="B1" s="9" t="s">
+        <v>3</v>
+      </c>
+      <c r="C1" s="9"/>
+      <c r="D1" s="9"/>
+      <c r="E1" s="9"/>
+      <c r="F1" s="9"/>
+      <c r="G1" s="9"/>
+      <c r="H1" s="9"/>
+      <c r="I1" s="9"/>
+      <c r="J1" s="9"/>
+      <c r="K1" s="9"/>
+      <c r="L1" s="9"/>
+      <c r="M1" s="10"/>
     </row>
     <row r="2" spans="1:13" s="2" customFormat="1" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A2" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="B2" s="8">
+      <c r="B2" s="12">
         <v>0.01</v>
       </c>
-      <c r="C2" s="9">
+      <c r="C2" s="13">
         <v>0.02</v>
       </c>
-      <c r="D2" s="9">
+      <c r="D2" s="13">
         <v>0.03</v>
       </c>
-      <c r="E2" s="9">
+      <c r="E2" s="13">
         <v>0.04</v>
       </c>
-      <c r="F2" s="9">
+      <c r="F2" s="13">
         <v>0.05</v>
       </c>
-      <c r="G2" s="9">
+      <c r="G2" s="13">
         <v>0.06</v>
       </c>
-      <c r="H2" s="9">
+      <c r="H2" s="13">
         <v>7.0000000000000007E-2</v>
       </c>
-      <c r="I2" s="9">
+      <c r="I2" s="13">
         <v>0.08</v>
       </c>
-      <c r="J2" s="9">
+      <c r="J2" s="13">
         <v>0.09</v>
       </c>
-      <c r="K2" s="9">
+      <c r="K2" s="13">
         <v>0.1</v>
       </c>
-      <c r="L2" s="9">
+      <c r="L2" s="13">
         <v>0.11</v>
       </c>
-      <c r="M2" s="10">
+      <c r="M2" s="14">
         <v>0.12</v>
       </c>
     </row>
@@ -727,708 +731,711 @@
       <c r="A3" s="5">
         <v>1</v>
       </c>
-      <c r="B3" s="11">
+      <c r="B3" s="8">
         <f>IF($B$1=Tabelle2!$A$1,(1+Tabelle1!B$2)^Tabelle1!$A3,IF($B$1=Tabelle2!$A$2,(1+Tabelle1!B$2)^(-Tabelle1!$A3),IF($B$1=Tabelle2!$A$3,((1+Tabelle1!B$2)^Tabelle1!$A3-1)/(Tabelle1!B$2*(1+Tabelle1!B$2)^Tabelle1!$A3),IF($B$1=Tabelle2!$A$4,(Tabelle1!B$2*(1+Tabelle1!B$2)^Tabelle1!$A3)/((1+Tabelle1!B$2)^Tabelle1!$A3-1)))))</f>
-        <v>0.99009900990099098</v>
-      </c>
-      <c r="C3" s="11">
+        <v>1.0099999999999991</v>
+      </c>
+      <c r="C3" s="8">
         <f>IF($B$1=Tabelle2!$A$1,(1+Tabelle1!C$2)^Tabelle1!$A3,IF($B$1=Tabelle2!$A$2,(1+Tabelle1!C$2)^(-Tabelle1!$A3),IF($B$1=Tabelle2!$A$3,((1+Tabelle1!C$2)^Tabelle1!$A3-1)/(Tabelle1!C$2*(1+Tabelle1!C$2)^Tabelle1!$A3),IF($B$1=Tabelle2!$A$4,(Tabelle1!C$2*(1+Tabelle1!C$2)^Tabelle1!$A3)/((1+Tabelle1!C$2)^Tabelle1!$A3-1)))))</f>
-        <v>0.98039215686274594</v>
-      </c>
-      <c r="D3" s="11">
+        <v>1.0199999999999991</v>
+      </c>
+      <c r="D3" s="8">
         <f>IF($B$1=Tabelle2!$A$1,(1+Tabelle1!D$2)^Tabelle1!$A3,IF($B$1=Tabelle2!$A$2,(1+Tabelle1!D$2)^(-Tabelle1!$A3),IF($B$1=Tabelle2!$A$3,((1+Tabelle1!D$2)^Tabelle1!$A3-1)/(Tabelle1!D$2*(1+Tabelle1!D$2)^Tabelle1!$A3),IF($B$1=Tabelle2!$A$4,(Tabelle1!D$2*(1+Tabelle1!D$2)^Tabelle1!$A3)/((1+Tabelle1!D$2)^Tabelle1!$A3-1)))))</f>
-        <v>0.97087378640776789</v>
-      </c>
-      <c r="E3" s="11">
+        <v>1.0299999999999991</v>
+      </c>
+      <c r="E3" s="8">
         <f>IF($B$1=Tabelle2!$A$1,(1+Tabelle1!E$2)^Tabelle1!$A3,IF($B$1=Tabelle2!$A$2,(1+Tabelle1!E$2)^(-Tabelle1!$A3),IF($B$1=Tabelle2!$A$3,((1+Tabelle1!E$2)^Tabelle1!$A3-1)/(Tabelle1!E$2*(1+Tabelle1!E$2)^Tabelle1!$A3),IF($B$1=Tabelle2!$A$4,(Tabelle1!E$2*(1+Tabelle1!E$2)^Tabelle1!$A3)/((1+Tabelle1!E$2)^Tabelle1!$A3-1)))))</f>
-        <v>0.96153846153846223</v>
-      </c>
-      <c r="F3" s="11">
+        <v>1.0399999999999991</v>
+      </c>
+      <c r="F3" s="8">
         <f>IF($B$1=Tabelle2!$A$1,(1+Tabelle1!F$2)^Tabelle1!$A3,IF($B$1=Tabelle2!$A$2,(1+Tabelle1!F$2)^(-Tabelle1!$A3),IF($B$1=Tabelle2!$A$3,((1+Tabelle1!F$2)^Tabelle1!$A3-1)/(Tabelle1!F$2*(1+Tabelle1!F$2)^Tabelle1!$A3),IF($B$1=Tabelle2!$A$4,(Tabelle1!F$2*(1+Tabelle1!F$2)^Tabelle1!$A3)/((1+Tabelle1!F$2)^Tabelle1!$A3-1)))))</f>
-        <v>0.95238095238095311</v>
-      </c>
-      <c r="G3" s="11">
+        <v>1.0499999999999992</v>
+      </c>
+      <c r="G3" s="8">
         <f>IF($B$1=Tabelle2!$A$1,(1+Tabelle1!G$2)^Tabelle1!$A3,IF($B$1=Tabelle2!$A$2,(1+Tabelle1!G$2)^(-Tabelle1!$A3),IF($B$1=Tabelle2!$A$3,((1+Tabelle1!G$2)^Tabelle1!$A3-1)/(Tabelle1!G$2*(1+Tabelle1!G$2)^Tabelle1!$A3),IF($B$1=Tabelle2!$A$4,(Tabelle1!G$2*(1+Tabelle1!G$2)^Tabelle1!$A3)/((1+Tabelle1!G$2)^Tabelle1!$A3-1)))))</f>
-        <v>0.94339622641509513</v>
-      </c>
-      <c r="H3" s="11">
+        <v>1.0599999999999992</v>
+      </c>
+      <c r="H3" s="8">
         <f>IF($B$1=Tabelle2!$A$1,(1+Tabelle1!H$2)^Tabelle1!$A3,IF($B$1=Tabelle2!$A$2,(1+Tabelle1!H$2)^(-Tabelle1!$A3),IF($B$1=Tabelle2!$A$3,((1+Tabelle1!H$2)^Tabelle1!$A3-1)/(Tabelle1!H$2*(1+Tabelle1!H$2)^Tabelle1!$A3),IF($B$1=Tabelle2!$A$4,(Tabelle1!H$2*(1+Tabelle1!H$2)^Tabelle1!$A3)/((1+Tabelle1!H$2)^Tabelle1!$A3-1)))))</f>
-        <v>0.93457943925233722</v>
-      </c>
-      <c r="I3" s="11">
+        <v>1.0699999999999992</v>
+      </c>
+      <c r="I3" s="8">
         <f>IF($B$1=Tabelle2!$A$1,(1+Tabelle1!I$2)^Tabelle1!$A3,IF($B$1=Tabelle2!$A$2,(1+Tabelle1!I$2)^(-Tabelle1!$A3),IF($B$1=Tabelle2!$A$3,((1+Tabelle1!I$2)^Tabelle1!$A3-1)/(Tabelle1!I$2*(1+Tabelle1!I$2)^Tabelle1!$A3),IF($B$1=Tabelle2!$A$4,(Tabelle1!I$2*(1+Tabelle1!I$2)^Tabelle1!$A3)/((1+Tabelle1!I$2)^Tabelle1!$A3-1)))))</f>
-        <v>0.92592592592592671</v>
-      </c>
-      <c r="J3" s="11">
+        <v>1.0799999999999992</v>
+      </c>
+      <c r="J3" s="8">
         <f>IF($B$1=Tabelle2!$A$1,(1+Tabelle1!J$2)^Tabelle1!$A3,IF($B$1=Tabelle2!$A$2,(1+Tabelle1!J$2)^(-Tabelle1!$A3),IF($B$1=Tabelle2!$A$3,((1+Tabelle1!J$2)^Tabelle1!$A3-1)/(Tabelle1!J$2*(1+Tabelle1!J$2)^Tabelle1!$A3),IF($B$1=Tabelle2!$A$4,(Tabelle1!J$2*(1+Tabelle1!J$2)^Tabelle1!$A3)/((1+Tabelle1!J$2)^Tabelle1!$A3-1)))))</f>
-        <v>0.91743119266055118</v>
-      </c>
-      <c r="K3" s="11">
+        <v>1.0899999999999992</v>
+      </c>
+      <c r="K3" s="8">
         <f>IF($B$1=Tabelle2!$A$1,(1+Tabelle1!K$2)^Tabelle1!$A3,IF($B$1=Tabelle2!$A$2,(1+Tabelle1!K$2)^(-Tabelle1!$A3),IF($B$1=Tabelle2!$A$3,((1+Tabelle1!K$2)^Tabelle1!$A3-1)/(Tabelle1!K$2*(1+Tabelle1!K$2)^Tabelle1!$A3),IF($B$1=Tabelle2!$A$4,(Tabelle1!K$2*(1+Tabelle1!K$2)^Tabelle1!$A3)/((1+Tabelle1!K$2)^Tabelle1!$A3-1)))))</f>
-        <v>0.90909090909090973</v>
-      </c>
-      <c r="L3" s="11">
+        <v>1.0999999999999992</v>
+      </c>
+      <c r="L3" s="8">
         <f>IF($B$1=Tabelle2!$A$1,(1+Tabelle1!L$2)^Tabelle1!$A3,IF($B$1=Tabelle2!$A$2,(1+Tabelle1!L$2)^(-Tabelle1!$A3),IF($B$1=Tabelle2!$A$3,((1+Tabelle1!L$2)^Tabelle1!$A3-1)/(Tabelle1!L$2*(1+Tabelle1!L$2)^Tabelle1!$A3),IF($B$1=Tabelle2!$A$4,(Tabelle1!L$2*(1+Tabelle1!L$2)^Tabelle1!$A3)/((1+Tabelle1!L$2)^Tabelle1!$A3-1)))))</f>
-        <v>0.90090090090090158</v>
-      </c>
-      <c r="M3" s="11">
+        <v>1.1099999999999992</v>
+      </c>
+      <c r="M3" s="8">
         <f>IF($B$1=Tabelle2!$A$1,(1+Tabelle1!M$2)^Tabelle1!$A3,IF($B$1=Tabelle2!$A$2,(1+Tabelle1!M$2)^(-Tabelle1!$A3),IF($B$1=Tabelle2!$A$3,((1+Tabelle1!M$2)^Tabelle1!$A3-1)/(Tabelle1!M$2*(1+Tabelle1!M$2)^Tabelle1!$A3),IF($B$1=Tabelle2!$A$4,(Tabelle1!M$2*(1+Tabelle1!M$2)^Tabelle1!$A3)/((1+Tabelle1!M$2)^Tabelle1!$A3-1)))))</f>
-        <v>0.89285714285714357</v>
+        <v>1.1199999999999992</v>
       </c>
     </row>
     <row r="4" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A4" s="6">
         <v>2</v>
       </c>
-      <c r="B4" s="11">
+      <c r="B4" s="8">
         <f>IF($B$1=Tabelle2!$A$1,(1+Tabelle1!B$2)^Tabelle1!$A4,IF($B$1=Tabelle2!$A$2,(1+Tabelle1!B$2)^(-Tabelle1!$A4),IF($B$1=Tabelle2!$A$3,((1+Tabelle1!B$2)^Tabelle1!$A4-1)/(Tabelle1!B$2*(1+Tabelle1!B$2)^Tabelle1!$A4),IF($B$1=Tabelle2!$A$4,(Tabelle1!B$2*(1+Tabelle1!B$2)^Tabelle1!$A4)/((1+Tabelle1!B$2)^Tabelle1!$A4-1)))))</f>
-        <v>1.9703950593079116</v>
-      </c>
-      <c r="C4" s="11">
+        <v>0.50751243781094513</v>
+      </c>
+      <c r="C4" s="8">
         <f>IF($B$1=Tabelle2!$A$1,(1+Tabelle1!C$2)^Tabelle1!$A4,IF($B$1=Tabelle2!$A$2,(1+Tabelle1!C$2)^(-Tabelle1!$A4),IF($B$1=Tabelle2!$A$3,((1+Tabelle1!C$2)^Tabelle1!$A4-1)/(Tabelle1!C$2*(1+Tabelle1!C$2)^Tabelle1!$A4),IF($B$1=Tabelle2!$A$4,(Tabelle1!C$2*(1+Tabelle1!C$2)^Tabelle1!$A4)/((1+Tabelle1!C$2)^Tabelle1!$A4-1)))))</f>
-        <v>1.9415609381007302</v>
-      </c>
-      <c r="D4" s="11">
+        <v>0.51504950495049517</v>
+      </c>
+      <c r="D4" s="8">
         <f>IF($B$1=Tabelle2!$A$1,(1+Tabelle1!D$2)^Tabelle1!$A4,IF($B$1=Tabelle2!$A$2,(1+Tabelle1!D$2)^(-Tabelle1!$A4),IF($B$1=Tabelle2!$A$3,((1+Tabelle1!D$2)^Tabelle1!$A4-1)/(Tabelle1!D$2*(1+Tabelle1!D$2)^Tabelle1!$A4),IF($B$1=Tabelle2!$A$4,(Tabelle1!D$2*(1+Tabelle1!D$2)^Tabelle1!$A4)/((1+Tabelle1!D$2)^Tabelle1!$A4-1)))))</f>
-        <v>1.9134696955415202</v>
-      </c>
-      <c r="E4" s="11">
+        <v>0.52261083743842396</v>
+      </c>
+      <c r="E4" s="8">
         <f>IF($B$1=Tabelle2!$A$1,(1+Tabelle1!E$2)^Tabelle1!$A4,IF($B$1=Tabelle2!$A$2,(1+Tabelle1!E$2)^(-Tabelle1!$A4),IF($B$1=Tabelle2!$A$3,((1+Tabelle1!E$2)^Tabelle1!$A4-1)/(Tabelle1!E$2*(1+Tabelle1!E$2)^Tabelle1!$A4),IF($B$1=Tabelle2!$A$4,(Tabelle1!E$2*(1+Tabelle1!E$2)^Tabelle1!$A4)/((1+Tabelle1!E$2)^Tabelle1!$A4-1)))))</f>
-        <v>1.8860946745562155</v>
-      </c>
-      <c r="F4" s="11">
+        <v>0.53019607843137184</v>
+      </c>
+      <c r="F4" s="8">
         <f>IF($B$1=Tabelle2!$A$1,(1+Tabelle1!F$2)^Tabelle1!$A4,IF($B$1=Tabelle2!$A$2,(1+Tabelle1!F$2)^(-Tabelle1!$A4),IF($B$1=Tabelle2!$A$3,((1+Tabelle1!F$2)^Tabelle1!$A4-1)/(Tabelle1!F$2*(1+Tabelle1!F$2)^Tabelle1!$A4),IF($B$1=Tabelle2!$A$4,(Tabelle1!F$2*(1+Tabelle1!F$2)^Tabelle1!$A4)/((1+Tabelle1!F$2)^Tabelle1!$A4-1)))))</f>
-        <v>1.8594104308390027</v>
-      </c>
-      <c r="G4" s="11">
+        <v>0.53780487804878041</v>
+      </c>
+      <c r="G4" s="8">
         <f>IF($B$1=Tabelle2!$A$1,(1+Tabelle1!G$2)^Tabelle1!$A4,IF($B$1=Tabelle2!$A$2,(1+Tabelle1!G$2)^(-Tabelle1!$A4),IF($B$1=Tabelle2!$A$3,((1+Tabelle1!G$2)^Tabelle1!$A4-1)/(Tabelle1!G$2*(1+Tabelle1!G$2)^Tabelle1!$A4),IF($B$1=Tabelle2!$A$4,(Tabelle1!G$2*(1+Tabelle1!G$2)^Tabelle1!$A4)/((1+Tabelle1!G$2)^Tabelle1!$A4-1)))))</f>
-        <v>1.8333926664293365</v>
-      </c>
-      <c r="H4" s="11">
+        <v>0.54543689320388289</v>
+      </c>
+      <c r="H4" s="8">
         <f>IF($B$1=Tabelle2!$A$1,(1+Tabelle1!H$2)^Tabelle1!$A4,IF($B$1=Tabelle2!$A$2,(1+Tabelle1!H$2)^(-Tabelle1!$A4),IF($B$1=Tabelle2!$A$3,((1+Tabelle1!H$2)^Tabelle1!$A4-1)/(Tabelle1!H$2*(1+Tabelle1!H$2)^Tabelle1!$A4),IF($B$1=Tabelle2!$A$4,(Tabelle1!H$2*(1+Tabelle1!H$2)^Tabelle1!$A4)/((1+Tabelle1!H$2)^Tabelle1!$A4-1)))))</f>
-        <v>1.8080181675255482</v>
-      </c>
-      <c r="I4" s="11">
+        <v>0.5530917874396134</v>
+      </c>
+      <c r="I4" s="8">
         <f>IF($B$1=Tabelle2!$A$1,(1+Tabelle1!I$2)^Tabelle1!$A4,IF($B$1=Tabelle2!$A$2,(1+Tabelle1!I$2)^(-Tabelle1!$A4),IF($B$1=Tabelle2!$A$3,((1+Tabelle1!I$2)^Tabelle1!$A4-1)/(Tabelle1!I$2*(1+Tabelle1!I$2)^Tabelle1!$A4),IF($B$1=Tabelle2!$A$4,(Tabelle1!I$2*(1+Tabelle1!I$2)^Tabelle1!$A4)/((1+Tabelle1!I$2)^Tabelle1!$A4-1)))))</f>
-        <v>1.7832647462277103</v>
-      </c>
-      <c r="J4" s="11">
+        <v>0.56076923076923046</v>
+      </c>
+      <c r="J4" s="8">
         <f>IF($B$1=Tabelle2!$A$1,(1+Tabelle1!J$2)^Tabelle1!$A4,IF($B$1=Tabelle2!$A$2,(1+Tabelle1!J$2)^(-Tabelle1!$A4),IF($B$1=Tabelle2!$A$3,((1+Tabelle1!J$2)^Tabelle1!$A4-1)/(Tabelle1!J$2*(1+Tabelle1!J$2)^Tabelle1!$A4),IF($B$1=Tabelle2!$A$4,(Tabelle1!J$2*(1+Tabelle1!J$2)^Tabelle1!$A4)/((1+Tabelle1!J$2)^Tabelle1!$A4-1)))))</f>
-        <v>1.7591111859271118</v>
-      </c>
-      <c r="K4" s="11">
+        <v>0.56846889952153068</v>
+      </c>
+      <c r="K4" s="8">
         <f>IF($B$1=Tabelle2!$A$1,(1+Tabelle1!K$2)^Tabelle1!$A4,IF($B$1=Tabelle2!$A$2,(1+Tabelle1!K$2)^(-Tabelle1!$A4),IF($B$1=Tabelle2!$A$3,((1+Tabelle1!K$2)^Tabelle1!$A4-1)/(Tabelle1!K$2*(1+Tabelle1!K$2)^Tabelle1!$A4),IF($B$1=Tabelle2!$A$4,(Tabelle1!K$2*(1+Tabelle1!K$2)^Tabelle1!$A4)/((1+Tabelle1!K$2)^Tabelle1!$A4-1)))))</f>
-        <v>1.7355371900826457</v>
-      </c>
-      <c r="L4" s="11">
+        <v>0.57619047619047581</v>
+      </c>
+      <c r="L4" s="8">
         <f>IF($B$1=Tabelle2!$A$1,(1+Tabelle1!L$2)^Tabelle1!$A4,IF($B$1=Tabelle2!$A$2,(1+Tabelle1!L$2)^(-Tabelle1!$A4),IF($B$1=Tabelle2!$A$3,((1+Tabelle1!L$2)^Tabelle1!$A4-1)/(Tabelle1!L$2*(1+Tabelle1!L$2)^Tabelle1!$A4),IF($B$1=Tabelle2!$A$4,(Tabelle1!L$2*(1+Tabelle1!L$2)^Tabelle1!$A4)/((1+Tabelle1!L$2)^Tabelle1!$A4-1)))))</f>
-        <v>1.7125233341449571</v>
-      </c>
-      <c r="M4" s="11">
+        <v>0.58393364928909908</v>
+      </c>
+      <c r="M4" s="8">
         <f>IF($B$1=Tabelle2!$A$1,(1+Tabelle1!M$2)^Tabelle1!$A4,IF($B$1=Tabelle2!$A$2,(1+Tabelle1!M$2)^(-Tabelle1!$A4),IF($B$1=Tabelle2!$A$3,((1+Tabelle1!M$2)^Tabelle1!$A4-1)/(Tabelle1!M$2*(1+Tabelle1!M$2)^Tabelle1!$A4),IF($B$1=Tabelle2!$A$4,(Tabelle1!M$2*(1+Tabelle1!M$2)^Tabelle1!$A4)/((1+Tabelle1!M$2)^Tabelle1!$A4-1)))))</f>
-        <v>1.6900510204081642</v>
+        <v>0.59169811320754684</v>
       </c>
     </row>
     <row r="5" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A5" s="6">
         <v>3</v>
       </c>
-      <c r="B5" s="11">
+      <c r="B5" s="8">
         <f>IF($B$1=Tabelle2!$A$1,(1+Tabelle1!B$2)^Tabelle1!$A5,IF($B$1=Tabelle2!$A$2,(1+Tabelle1!B$2)^(-Tabelle1!$A5),IF($B$1=Tabelle2!$A$3,((1+Tabelle1!B$2)^Tabelle1!$A5-1)/(Tabelle1!B$2*(1+Tabelle1!B$2)^Tabelle1!$A5),IF($B$1=Tabelle2!$A$4,(Tabelle1!B$2*(1+Tabelle1!B$2)^Tabelle1!$A5)/((1+Tabelle1!B$2)^Tabelle1!$A5-1)))))</f>
-        <v>2.9409852072355469</v>
-      </c>
-      <c r="C5" s="11">
+        <v>0.34002211148147021</v>
+      </c>
+      <c r="C5" s="8">
         <f>IF($B$1=Tabelle2!$A$1,(1+Tabelle1!C$2)^Tabelle1!$A5,IF($B$1=Tabelle2!$A$2,(1+Tabelle1!C$2)^(-Tabelle1!$A5),IF($B$1=Tabelle2!$A$3,((1+Tabelle1!C$2)^Tabelle1!$A5-1)/(Tabelle1!C$2*(1+Tabelle1!C$2)^Tabelle1!$A5),IF($B$1=Tabelle2!$A$4,(Tabelle1!C$2*(1+Tabelle1!C$2)^Tabelle1!$A5)/((1+Tabelle1!C$2)^Tabelle1!$A5-1)))))</f>
-        <v>2.8838832726477719</v>
-      </c>
-      <c r="D5" s="11">
+        <v>0.34675467259181847</v>
+      </c>
+      <c r="D5" s="8">
         <f>IF($B$1=Tabelle2!$A$1,(1+Tabelle1!D$2)^Tabelle1!$A5,IF($B$1=Tabelle2!$A$2,(1+Tabelle1!D$2)^(-Tabelle1!$A5),IF($B$1=Tabelle2!$A$3,((1+Tabelle1!D$2)^Tabelle1!$A5-1)/(Tabelle1!D$2*(1+Tabelle1!D$2)^Tabelle1!$A5),IF($B$1=Tabelle2!$A$4,(Tabelle1!D$2*(1+Tabelle1!D$2)^Tabelle1!$A5)/((1+Tabelle1!D$2)^Tabelle1!$A5-1)))))</f>
-        <v>2.8286113548946807</v>
-      </c>
-      <c r="E5" s="11">
+        <v>0.35353036332459803</v>
+      </c>
+      <c r="E5" s="8">
         <f>IF($B$1=Tabelle2!$A$1,(1+Tabelle1!E$2)^Tabelle1!$A5,IF($B$1=Tabelle2!$A$2,(1+Tabelle1!E$2)^(-Tabelle1!$A5),IF($B$1=Tabelle2!$A$3,((1+Tabelle1!E$2)^Tabelle1!$A5-1)/(Tabelle1!E$2*(1+Tabelle1!E$2)^Tabelle1!$A5),IF($B$1=Tabelle2!$A$4,(Tabelle1!E$2*(1+Tabelle1!E$2)^Tabelle1!$A5)/((1+Tabelle1!E$2)^Tabelle1!$A5-1)))))</f>
-        <v>2.7750910332271297</v>
-      </c>
-      <c r="F5" s="11">
+        <v>0.36034853921066096</v>
+      </c>
+      <c r="F5" s="8">
         <f>IF($B$1=Tabelle2!$A$1,(1+Tabelle1!F$2)^Tabelle1!$A5,IF($B$1=Tabelle2!$A$2,(1+Tabelle1!F$2)^(-Tabelle1!$A5),IF($B$1=Tabelle2!$A$3,((1+Tabelle1!F$2)^Tabelle1!$A5-1)/(Tabelle1!F$2*(1+Tabelle1!F$2)^Tabelle1!$A5),IF($B$1=Tabelle2!$A$4,(Tabelle1!F$2*(1+Tabelle1!F$2)^Tabelle1!$A5)/((1+Tabelle1!F$2)^Tabelle1!$A5-1)))))</f>
-        <v>2.7232480293704802</v>
-      </c>
-      <c r="G5" s="11">
+        <v>0.36720856463124479</v>
+      </c>
+      <c r="G5" s="8">
         <f>IF($B$1=Tabelle2!$A$1,(1+Tabelle1!G$2)^Tabelle1!$A5,IF($B$1=Tabelle2!$A$2,(1+Tabelle1!G$2)^(-Tabelle1!$A5),IF($B$1=Tabelle2!$A$3,((1+Tabelle1!G$2)^Tabelle1!$A5-1)/(Tabelle1!G$2*(1+Tabelle1!G$2)^Tabelle1!$A5),IF($B$1=Tabelle2!$A$4,(Tabelle1!G$2*(1+Tabelle1!G$2)^Tabelle1!$A5)/((1+Tabelle1!G$2)^Tabelle1!$A5-1)))))</f>
-        <v>2.6730119494616398</v>
-      </c>
-      <c r="H5" s="11">
+        <v>0.37410981279055111</v>
+      </c>
+      <c r="H5" s="8">
         <f>IF($B$1=Tabelle2!$A$1,(1+Tabelle1!H$2)^Tabelle1!$A5,IF($B$1=Tabelle2!$A$2,(1+Tabelle1!H$2)^(-Tabelle1!$A5),IF($B$1=Tabelle2!$A$3,((1+Tabelle1!H$2)^Tabelle1!$A5-1)/(Tabelle1!H$2*(1+Tabelle1!H$2)^Tabelle1!$A5),IF($B$1=Tabelle2!$A$4,(Tabelle1!H$2*(1+Tabelle1!H$2)^Tabelle1!$A5)/((1+Tabelle1!H$2)^Tabelle1!$A5-1)))))</f>
-        <v>2.6243160444164007</v>
-      </c>
-      <c r="I5" s="11">
+        <v>0.38105166568166965</v>
+      </c>
+      <c r="I5" s="8">
         <f>IF($B$1=Tabelle2!$A$1,(1+Tabelle1!I$2)^Tabelle1!$A5,IF($B$1=Tabelle2!$A$2,(1+Tabelle1!I$2)^(-Tabelle1!$A5),IF($B$1=Tabelle2!$A$3,((1+Tabelle1!I$2)^Tabelle1!$A5-1)/(Tabelle1!I$2*(1+Tabelle1!I$2)^Tabelle1!$A5),IF($B$1=Tabelle2!$A$4,(Tabelle1!I$2*(1+Tabelle1!I$2)^Tabelle1!$A5)/((1+Tabelle1!I$2)^Tabelle1!$A5-1)))))</f>
-        <v>2.5770969872478804</v>
-      </c>
-      <c r="J5" s="11">
+        <v>0.38803351404632802</v>
+      </c>
+      <c r="J5" s="8">
         <f>IF($B$1=Tabelle2!$A$1,(1+Tabelle1!J$2)^Tabelle1!$A5,IF($B$1=Tabelle2!$A$2,(1+Tabelle1!J$2)^(-Tabelle1!$A5),IF($B$1=Tabelle2!$A$3,((1+Tabelle1!J$2)^Tabelle1!$A5-1)/(Tabelle1!J$2*(1+Tabelle1!J$2)^Tabelle1!$A5),IF($B$1=Tabelle2!$A$4,(Tabelle1!J$2*(1+Tabelle1!J$2)^Tabelle1!$A5)/((1+Tabelle1!J$2)^Tabelle1!$A5-1)))))</f>
-        <v>2.5312946659881761</v>
-      </c>
-      <c r="K5" s="11">
+        <v>0.3950547573289403</v>
+      </c>
+      <c r="K5" s="8">
         <f>IF($B$1=Tabelle2!$A$1,(1+Tabelle1!K$2)^Tabelle1!$A5,IF($B$1=Tabelle2!$A$2,(1+Tabelle1!K$2)^(-Tabelle1!$A5),IF($B$1=Tabelle2!$A$3,((1+Tabelle1!K$2)^Tabelle1!$A5-1)/(Tabelle1!K$2*(1+Tabelle1!K$2)^Tabelle1!$A5),IF($B$1=Tabelle2!$A$4,(Tabelle1!K$2*(1+Tabelle1!K$2)^Tabelle1!$A5)/((1+Tabelle1!K$2)^Tabelle1!$A5-1)))))</f>
-        <v>2.4868519909842246</v>
-      </c>
-      <c r="L5" s="11">
+        <v>0.40211480362537733</v>
+      </c>
+      <c r="L5" s="8">
         <f>IF($B$1=Tabelle2!$A$1,(1+Tabelle1!L$2)^Tabelle1!$A5,IF($B$1=Tabelle2!$A$2,(1+Tabelle1!L$2)^(-Tabelle1!$A5),IF($B$1=Tabelle2!$A$3,((1+Tabelle1!L$2)^Tabelle1!$A5-1)/(Tabelle1!L$2*(1+Tabelle1!L$2)^Tabelle1!$A5),IF($B$1=Tabelle2!$A$4,(Tabelle1!L$2*(1+Tabelle1!L$2)^Tabelle1!$A5)/((1+Tabelle1!L$2)^Tabelle1!$A5-1)))))</f>
-        <v>2.4437147154459073</v>
-      </c>
-      <c r="M5" s="11">
+        <v>0.40921306962688109</v>
+      </c>
+      <c r="M5" s="8">
         <f>IF($B$1=Tabelle2!$A$1,(1+Tabelle1!M$2)^Tabelle1!$A5,IF($B$1=Tabelle2!$A$2,(1+Tabelle1!M$2)^(-Tabelle1!$A5),IF($B$1=Tabelle2!$A$3,((1+Tabelle1!M$2)^Tabelle1!$A5-1)/(Tabelle1!M$2*(1+Tabelle1!M$2)^Tabelle1!$A5),IF($B$1=Tabelle2!$A$4,(Tabelle1!M$2*(1+Tabelle1!M$2)^Tabelle1!$A5)/((1+Tabelle1!M$2)^Tabelle1!$A5-1)))))</f>
-        <v>2.4018312682215761</v>
+        <v>0.41634898055950659</v>
       </c>
     </row>
     <row r="6" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A6" s="6">
         <v>4</v>
       </c>
-      <c r="B6" s="11">
+      <c r="B6" s="8">
         <f>IF($B$1=Tabelle2!$A$1,(1+Tabelle1!B$2)^Tabelle1!$A6,IF($B$1=Tabelle2!$A$2,(1+Tabelle1!B$2)^(-Tabelle1!$A6),IF($B$1=Tabelle2!$A$3,((1+Tabelle1!B$2)^Tabelle1!$A6-1)/(Tabelle1!B$2*(1+Tabelle1!B$2)^Tabelle1!$A6),IF($B$1=Tabelle2!$A$4,(Tabelle1!B$2*(1+Tabelle1!B$2)^Tabelle1!$A6)/((1+Tabelle1!B$2)^Tabelle1!$A6-1)))))</f>
-        <v>3.9019655517183742</v>
-      </c>
-      <c r="C6" s="11">
+        <v>0.25628109391166032</v>
+      </c>
+      <c r="C6" s="8">
         <f>IF($B$1=Tabelle2!$A$1,(1+Tabelle1!C$2)^Tabelle1!$A6,IF($B$1=Tabelle2!$A$2,(1+Tabelle1!C$2)^(-Tabelle1!$A6),IF($B$1=Tabelle2!$A$3,((1+Tabelle1!C$2)^Tabelle1!$A6-1)/(Tabelle1!C$2*(1+Tabelle1!C$2)^Tabelle1!$A6),IF($B$1=Tabelle2!$A$4,(Tabelle1!C$2*(1+Tabelle1!C$2)^Tabelle1!$A6)/((1+Tabelle1!C$2)^Tabelle1!$A6-1)))))</f>
-        <v>3.8077286986742878</v>
-      </c>
-      <c r="D6" s="11">
+        <v>0.26262375267128762</v>
+      </c>
+      <c r="D6" s="8">
         <f>IF($B$1=Tabelle2!$A$1,(1+Tabelle1!D$2)^Tabelle1!$A6,IF($B$1=Tabelle2!$A$2,(1+Tabelle1!D$2)^(-Tabelle1!$A6),IF($B$1=Tabelle2!$A$3,((1+Tabelle1!D$2)^Tabelle1!$A6-1)/(Tabelle1!D$2*(1+Tabelle1!D$2)^Tabelle1!$A6),IF($B$1=Tabelle2!$A$4,(Tabelle1!D$2*(1+Tabelle1!D$2)^Tabelle1!$A6)/((1+Tabelle1!D$2)^Tabelle1!$A6-1)))))</f>
-        <v>3.7170984028103682</v>
-      </c>
-      <c r="E6" s="11">
+        <v>0.26902704519308257</v>
+      </c>
+      <c r="E6" s="8">
         <f>IF($B$1=Tabelle2!$A$1,(1+Tabelle1!E$2)^Tabelle1!$A6,IF($B$1=Tabelle2!$A$2,(1+Tabelle1!E$2)^(-Tabelle1!$A6),IF($B$1=Tabelle2!$A$3,((1+Tabelle1!E$2)^Tabelle1!$A6-1)/(Tabelle1!E$2*(1+Tabelle1!E$2)^Tabelle1!$A6),IF($B$1=Tabelle2!$A$4,(Tabelle1!E$2*(1+Tabelle1!E$2)^Tabelle1!$A6)/((1+Tabelle1!E$2)^Tabelle1!$A6-1)))))</f>
-        <v>3.6298952242568578</v>
-      </c>
-      <c r="F6" s="11">
+        <v>0.27549004536480204</v>
+      </c>
+      <c r="F6" s="8">
         <f>IF($B$1=Tabelle2!$A$1,(1+Tabelle1!F$2)^Tabelle1!$A6,IF($B$1=Tabelle2!$A$2,(1+Tabelle1!F$2)^(-Tabelle1!$A6),IF($B$1=Tabelle2!$A$3,((1+Tabelle1!F$2)^Tabelle1!$A6-1)/(Tabelle1!F$2*(1+Tabelle1!F$2)^Tabelle1!$A6),IF($B$1=Tabelle2!$A$4,(Tabelle1!F$2*(1+Tabelle1!F$2)^Tabelle1!$A6)/((1+Tabelle1!F$2)^Tabelle1!$A6-1)))))</f>
-        <v>3.5459505041623602</v>
-      </c>
-      <c r="G6" s="11">
+        <v>0.2820118326034628</v>
+      </c>
+      <c r="G6" s="8">
         <f>IF($B$1=Tabelle2!$A$1,(1+Tabelle1!G$2)^Tabelle1!$A6,IF($B$1=Tabelle2!$A$2,(1+Tabelle1!G$2)^(-Tabelle1!$A6),IF($B$1=Tabelle2!$A$3,((1+Tabelle1!G$2)^Tabelle1!$A6-1)/(Tabelle1!G$2*(1+Tabelle1!G$2)^Tabelle1!$A6),IF($B$1=Tabelle2!$A$4,(Tabelle1!G$2*(1+Tabelle1!G$2)^Tabelle1!$A6)/((1+Tabelle1!G$2)^Tabelle1!$A6-1)))))</f>
-        <v>3.4651056126996602</v>
-      </c>
-      <c r="H6" s="11">
+        <v>0.28859149237327314</v>
+      </c>
+      <c r="H6" s="8">
         <f>IF($B$1=Tabelle2!$A$1,(1+Tabelle1!H$2)^Tabelle1!$A6,IF($B$1=Tabelle2!$A$2,(1+Tabelle1!H$2)^(-Tabelle1!$A6),IF($B$1=Tabelle2!$A$3,((1+Tabelle1!H$2)^Tabelle1!$A6-1)/(Tabelle1!H$2*(1+Tabelle1!H$2)^Tabelle1!$A6),IF($B$1=Tabelle2!$A$4,(Tabelle1!H$2*(1+Tabelle1!H$2)^Tabelle1!$A6)/((1+Tabelle1!H$2)^Tabelle1!$A6-1)))))</f>
-        <v>3.387211256463925</v>
-      </c>
-      <c r="I6" s="11">
+        <v>0.29522811666726356</v>
+      </c>
+      <c r="I6" s="8">
         <f>IF($B$1=Tabelle2!$A$1,(1+Tabelle1!I$2)^Tabelle1!$A6,IF($B$1=Tabelle2!$A$2,(1+Tabelle1!I$2)^(-Tabelle1!$A6),IF($B$1=Tabelle2!$A$3,((1+Tabelle1!I$2)^Tabelle1!$A6-1)/(Tabelle1!I$2*(1+Tabelle1!I$2)^Tabelle1!$A6),IF($B$1=Tabelle2!$A$4,(Tabelle1!I$2*(1+Tabelle1!I$2)^Tabelle1!$A6)/((1+Tabelle1!I$2)^Tabelle1!$A6-1)))))</f>
-        <v>3.3121268400443342</v>
-      </c>
-      <c r="J6" s="11">
+        <v>0.30192080445403913</v>
+      </c>
+      <c r="J6" s="8">
         <f>IF($B$1=Tabelle2!$A$1,(1+Tabelle1!J$2)^Tabelle1!$A6,IF($B$1=Tabelle2!$A$2,(1+Tabelle1!J$2)^(-Tabelle1!$A6),IF($B$1=Tabelle2!$A$3,((1+Tabelle1!J$2)^Tabelle1!$A6-1)/(Tabelle1!J$2*(1+Tabelle1!J$2)^Tabelle1!$A6),IF($B$1=Tabelle2!$A$4,(Tabelle1!J$2*(1+Tabelle1!J$2)^Tabelle1!$A6)/((1+Tabelle1!J$2)^Tabelle1!$A6-1)))))</f>
-        <v>3.2397198770533731</v>
-      </c>
-      <c r="K6" s="11">
+        <v>0.30866866209109767</v>
+      </c>
+      <c r="K6" s="8">
         <f>IF($B$1=Tabelle2!$A$1,(1+Tabelle1!K$2)^Tabelle1!$A6,IF($B$1=Tabelle2!$A$2,(1+Tabelle1!K$2)^(-Tabelle1!$A6),IF($B$1=Tabelle2!$A$3,((1+Tabelle1!K$2)^Tabelle1!$A6-1)/(Tabelle1!K$2*(1+Tabelle1!K$2)^Tabelle1!$A6),IF($B$1=Tabelle2!$A$4,(Tabelle1!K$2*(1+Tabelle1!K$2)^Tabelle1!$A6)/((1+Tabelle1!K$2)^Tabelle1!$A6-1)))))</f>
-        <v>3.169865446349295</v>
-      </c>
-      <c r="L6" s="11">
+        <v>0.31547080370609765</v>
+      </c>
+      <c r="L6" s="8">
         <f>IF($B$1=Tabelle2!$A$1,(1+Tabelle1!L$2)^Tabelle1!$A6,IF($B$1=Tabelle2!$A$2,(1+Tabelle1!L$2)^(-Tabelle1!$A6),IF($B$1=Tabelle2!$A$3,((1+Tabelle1!L$2)^Tabelle1!$A6-1)/(Tabelle1!L$2*(1+Tabelle1!L$2)^Tabelle1!$A6),IF($B$1=Tabelle2!$A$4,(Tabelle1!L$2*(1+Tabelle1!L$2)^Tabelle1!$A6)/((1+Tabelle1!L$2)^Tabelle1!$A6-1)))))</f>
-        <v>3.1024456895909078</v>
-      </c>
-      <c r="M6" s="11">
+        <v>0.32232635154746614</v>
+      </c>
+      <c r="M6" s="8">
         <f>IF($B$1=Tabelle2!$A$1,(1+Tabelle1!M$2)^Tabelle1!$A6,IF($B$1=Tabelle2!$A$2,(1+Tabelle1!M$2)^(-Tabelle1!$A6),IF($B$1=Tabelle2!$A$3,((1+Tabelle1!M$2)^Tabelle1!$A6-1)/(Tabelle1!M$2*(1+Tabelle1!M$2)^Tabelle1!$A6),IF($B$1=Tabelle2!$A$4,(Tabelle1!M$2*(1+Tabelle1!M$2)^Tabelle1!$A6)/((1+Tabelle1!M$2)^Tabelle1!$A6-1)))))</f>
-        <v>3.037349346626407</v>
+        <v>0.32923443630568966</v>
       </c>
     </row>
     <row r="7" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A7" s="6">
         <v>5</v>
       </c>
-      <c r="B7" s="11">
+      <c r="B7" s="8">
         <f>IF($B$1=Tabelle2!$A$1,(1+Tabelle1!B$2)^Tabelle1!$A7,IF($B$1=Tabelle2!$A$2,(1+Tabelle1!B$2)^(-Tabelle1!$A7),IF($B$1=Tabelle2!$A$3,((1+Tabelle1!B$2)^Tabelle1!$A7-1)/(Tabelle1!B$2*(1+Tabelle1!B$2)^Tabelle1!$A7),IF($B$1=Tabelle2!$A$4,(Tabelle1!B$2*(1+Tabelle1!B$2)^Tabelle1!$A7)/((1+Tabelle1!B$2)^Tabelle1!$A7-1)))))</f>
-        <v>4.853431239325114</v>
-      </c>
-      <c r="C7" s="11">
+        <v>0.20603979961588031</v>
+      </c>
+      <c r="C7" s="8">
         <f>IF($B$1=Tabelle2!$A$1,(1+Tabelle1!C$2)^Tabelle1!$A7,IF($B$1=Tabelle2!$A$2,(1+Tabelle1!C$2)^(-Tabelle1!$A7),IF($B$1=Tabelle2!$A$3,((1+Tabelle1!C$2)^Tabelle1!$A7-1)/(Tabelle1!C$2*(1+Tabelle1!C$2)^Tabelle1!$A7),IF($B$1=Tabelle2!$A$4,(Tabelle1!C$2*(1+Tabelle1!C$2)^Tabelle1!$A7)/((1+Tabelle1!C$2)^Tabelle1!$A7-1)))))</f>
-        <v>4.7134595085042053</v>
-      </c>
-      <c r="D7" s="11">
+        <v>0.21215839410432219</v>
+      </c>
+      <c r="D7" s="8">
         <f>IF($B$1=Tabelle2!$A$1,(1+Tabelle1!D$2)^Tabelle1!$A7,IF($B$1=Tabelle2!$A$2,(1+Tabelle1!D$2)^(-Tabelle1!$A7),IF($B$1=Tabelle2!$A$3,((1+Tabelle1!D$2)^Tabelle1!$A7-1)/(Tabelle1!D$2*(1+Tabelle1!D$2)^Tabelle1!$A7),IF($B$1=Tabelle2!$A$4,(Tabelle1!D$2*(1+Tabelle1!D$2)^Tabelle1!$A7)/((1+Tabelle1!D$2)^Tabelle1!$A7-1)))))</f>
-        <v>4.5797071871945301</v>
-      </c>
-      <c r="E7" s="11">
+        <v>0.21835457140057621</v>
+      </c>
+      <c r="E7" s="8">
         <f>IF($B$1=Tabelle2!$A$1,(1+Tabelle1!E$2)^Tabelle1!$A7,IF($B$1=Tabelle2!$A$2,(1+Tabelle1!E$2)^(-Tabelle1!$A7),IF($B$1=Tabelle2!$A$3,((1+Tabelle1!E$2)^Tabelle1!$A7-1)/(Tabelle1!E$2*(1+Tabelle1!E$2)^Tabelle1!$A7),IF($B$1=Tabelle2!$A$4,(Tabelle1!E$2*(1+Tabelle1!E$2)^Tabelle1!$A7)/((1+Tabelle1!E$2)^Tabelle1!$A7-1)))))</f>
-        <v>4.4518223310162108</v>
-      </c>
-      <c r="F7" s="11">
+        <v>0.22462711349303363</v>
+      </c>
+      <c r="F7" s="8">
         <f>IF($B$1=Tabelle2!$A$1,(1+Tabelle1!F$2)^Tabelle1!$A7,IF($B$1=Tabelle2!$A$2,(1+Tabelle1!F$2)^(-Tabelle1!$A7),IF($B$1=Tabelle2!$A$3,((1+Tabelle1!F$2)^Tabelle1!$A7-1)/(Tabelle1!F$2*(1+Tabelle1!F$2)^Tabelle1!$A7),IF($B$1=Tabelle2!$A$4,(Tabelle1!F$2*(1+Tabelle1!F$2)^Tabelle1!$A7)/((1+Tabelle1!F$2)^Tabelle1!$A7-1)))))</f>
-        <v>4.3294766706308208</v>
-      </c>
-      <c r="G7" s="11">
+        <v>0.23097479812826807</v>
+      </c>
+      <c r="G7" s="8">
         <f>IF($B$1=Tabelle2!$A$1,(1+Tabelle1!G$2)^Tabelle1!$A7,IF($B$1=Tabelle2!$A$2,(1+Tabelle1!G$2)^(-Tabelle1!$A7),IF($B$1=Tabelle2!$A$3,((1+Tabelle1!G$2)^Tabelle1!$A7-1)/(Tabelle1!G$2*(1+Tabelle1!G$2)^Tabelle1!$A7),IF($B$1=Tabelle2!$A$4,(Tabelle1!G$2*(1+Tabelle1!G$2)^Tabelle1!$A7)/((1+Tabelle1!G$2)^Tabelle1!$A7-1)))))</f>
-        <v>4.2123637855657181</v>
-      </c>
-      <c r="H7" s="11">
+        <v>0.23739640043118937</v>
+      </c>
+      <c r="H7" s="8">
         <f>IF($B$1=Tabelle2!$A$1,(1+Tabelle1!H$2)^Tabelle1!$A7,IF($B$1=Tabelle2!$A$2,(1+Tabelle1!H$2)^(-Tabelle1!$A7),IF($B$1=Tabelle2!$A$3,((1+Tabelle1!H$2)^Tabelle1!$A7-1)/(Tabelle1!H$2*(1+Tabelle1!H$2)^Tabelle1!$A7),IF($B$1=Tabelle2!$A$4,(Tabelle1!H$2*(1+Tabelle1!H$2)^Tabelle1!$A7)/((1+Tabelle1!H$2)^Tabelle1!$A7-1)))))</f>
-        <v>4.100197435947595</v>
-      </c>
-      <c r="I7" s="11">
+        <v>0.24389069444137401</v>
+      </c>
+      <c r="I7" s="8">
         <f>IF($B$1=Tabelle2!$A$1,(1+Tabelle1!I$2)^Tabelle1!$A7,IF($B$1=Tabelle2!$A$2,(1+Tabelle1!I$2)^(-Tabelle1!$A7),IF($B$1=Tabelle2!$A$3,((1+Tabelle1!I$2)^Tabelle1!$A7-1)/(Tabelle1!I$2*(1+Tabelle1!I$2)^Tabelle1!$A7),IF($B$1=Tabelle2!$A$4,(Tabelle1!I$2*(1+Tabelle1!I$2)^Tabelle1!$A7)/((1+Tabelle1!I$2)^Tabelle1!$A7-1)))))</f>
-        <v>3.9927100370780875</v>
-      </c>
-      <c r="J7" s="11">
+        <v>0.25045645456683646</v>
+      </c>
+      <c r="J7" s="8">
         <f>IF($B$1=Tabelle2!$A$1,(1+Tabelle1!J$2)^Tabelle1!$A7,IF($B$1=Tabelle2!$A$2,(1+Tabelle1!J$2)^(-Tabelle1!$A7),IF($B$1=Tabelle2!$A$3,((1+Tabelle1!J$2)^Tabelle1!$A7-1)/(Tabelle1!J$2*(1+Tabelle1!J$2)^Tabelle1!$A7),IF($B$1=Tabelle2!$A$4,(Tabelle1!J$2*(1+Tabelle1!J$2)^Tabelle1!$A7)/((1+Tabelle1!J$2)^Tabelle1!$A7-1)))))</f>
-        <v>3.8896512633517188</v>
-      </c>
-      <c r="K7" s="11">
+        <v>0.25709245695674482</v>
+      </c>
+      <c r="K7" s="8">
         <f>IF($B$1=Tabelle2!$A$1,(1+Tabelle1!K$2)^Tabelle1!$A7,IF($B$1=Tabelle2!$A$2,(1+Tabelle1!K$2)^(-Tabelle1!$A7),IF($B$1=Tabelle2!$A$3,((1+Tabelle1!K$2)^Tabelle1!$A7-1)/(Tabelle1!K$2*(1+Tabelle1!K$2)^Tabelle1!$A7),IF($B$1=Tabelle2!$A$4,(Tabelle1!K$2*(1+Tabelle1!K$2)^Tabelle1!$A7)/((1+Tabelle1!K$2)^Tabelle1!$A7-1)))))</f>
-        <v>3.7907867694084505</v>
-      </c>
-      <c r="L7" s="11">
+        <v>0.26379748079474524</v>
+      </c>
+      <c r="L7" s="8">
         <f>IF($B$1=Tabelle2!$A$1,(1+Tabelle1!L$2)^Tabelle1!$A7,IF($B$1=Tabelle2!$A$2,(1+Tabelle1!L$2)^(-Tabelle1!$A7),IF($B$1=Tabelle2!$A$3,((1+Tabelle1!L$2)^Tabelle1!$A7-1)/(Tabelle1!L$2*(1+Tabelle1!L$2)^Tabelle1!$A7),IF($B$1=Tabelle2!$A$4,(Tabelle1!L$2*(1+Tabelle1!L$2)^Tabelle1!$A7)/((1+Tabelle1!L$2)^Tabelle1!$A7-1)))))</f>
-        <v>3.6958970176494668</v>
-      </c>
-      <c r="M7" s="11">
+        <v>0.27057030951473438</v>
+      </c>
+      <c r="M7" s="8">
         <f>IF($B$1=Tabelle2!$A$1,(1+Tabelle1!M$2)^Tabelle1!$A7,IF($B$1=Tabelle2!$A$2,(1+Tabelle1!M$2)^(-Tabelle1!$A7),IF($B$1=Tabelle2!$A$3,((1+Tabelle1!M$2)^Tabelle1!$A7-1)/(Tabelle1!M$2*(1+Tabelle1!M$2)^Tabelle1!$A7),IF($B$1=Tabelle2!$A$4,(Tabelle1!M$2*(1+Tabelle1!M$2)^Tabelle1!$A7)/((1+Tabelle1!M$2)^Tabelle1!$A7-1)))))</f>
-        <v>3.6047762023450067</v>
+        <v>0.27740973194104873</v>
       </c>
     </row>
     <row r="8" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A8" s="6">
         <v>6</v>
       </c>
-      <c r="B8" s="11">
+      <c r="B8" s="8">
         <f>IF($B$1=Tabelle2!$A$1,(1+Tabelle1!B$2)^Tabelle1!$A8,IF($B$1=Tabelle2!$A$2,(1+Tabelle1!B$2)^(-Tabelle1!$A8),IF($B$1=Tabelle2!$A$3,((1+Tabelle1!B$2)^Tabelle1!$A8-1)/(Tabelle1!B$2*(1+Tabelle1!B$2)^Tabelle1!$A8),IF($B$1=Tabelle2!$A$4,(Tabelle1!B$2*(1+Tabelle1!B$2)^Tabelle1!$A8)/((1+Tabelle1!B$2)^Tabelle1!$A8-1)))))</f>
-        <v>5.7954764745793392</v>
-      </c>
-      <c r="C8" s="11">
+        <v>0.17254836671088106</v>
+      </c>
+      <c r="C8" s="8">
         <f>IF($B$1=Tabelle2!$A$1,(1+Tabelle1!C$2)^Tabelle1!$A8,IF($B$1=Tabelle2!$A$2,(1+Tabelle1!C$2)^(-Tabelle1!$A8),IF($B$1=Tabelle2!$A$3,((1+Tabelle1!C$2)^Tabelle1!$A8-1)/(Tabelle1!C$2*(1+Tabelle1!C$2)^Tabelle1!$A8),IF($B$1=Tabelle2!$A$4,(Tabelle1!C$2*(1+Tabelle1!C$2)^Tabelle1!$A8)/((1+Tabelle1!C$2)^Tabelle1!$A8-1)))))</f>
-        <v>5.6014308906904002</v>
-      </c>
-      <c r="D8" s="11">
+        <v>0.1785258123352024</v>
+      </c>
+      <c r="D8" s="8">
         <f>IF($B$1=Tabelle2!$A$1,(1+Tabelle1!D$2)^Tabelle1!$A8,IF($B$1=Tabelle2!$A$2,(1+Tabelle1!D$2)^(-Tabelle1!$A8),IF($B$1=Tabelle2!$A$3,((1+Tabelle1!D$2)^Tabelle1!$A8-1)/(Tabelle1!D$2*(1+Tabelle1!D$2)^Tabelle1!$A8),IF($B$1=Tabelle2!$A$4,(Tabelle1!D$2*(1+Tabelle1!D$2)^Tabelle1!$A8)/((1+Tabelle1!D$2)^Tabelle1!$A8-1)))))</f>
-        <v>5.4171914438781865</v>
-      </c>
-      <c r="E8" s="11">
+        <v>0.18459750045017728</v>
+      </c>
+      <c r="E8" s="8">
         <f>IF($B$1=Tabelle2!$A$1,(1+Tabelle1!E$2)^Tabelle1!$A8,IF($B$1=Tabelle2!$A$2,(1+Tabelle1!E$2)^(-Tabelle1!$A8),IF($B$1=Tabelle2!$A$3,((1+Tabelle1!E$2)^Tabelle1!$A8-1)/(Tabelle1!E$2*(1+Tabelle1!E$2)^Tabelle1!$A8),IF($B$1=Tabelle2!$A$4,(Tabelle1!E$2*(1+Tabelle1!E$2)^Tabelle1!$A8)/((1+Tabelle1!E$2)^Tabelle1!$A8-1)))))</f>
-        <v>5.2421368567463569</v>
-      </c>
-      <c r="F8" s="11">
+        <v>0.1907619025079538</v>
+      </c>
+      <c r="F8" s="8">
         <f>IF($B$1=Tabelle2!$A$1,(1+Tabelle1!F$2)^Tabelle1!$A8,IF($B$1=Tabelle2!$A$2,(1+Tabelle1!F$2)^(-Tabelle1!$A8),IF($B$1=Tabelle2!$A$3,((1+Tabelle1!F$2)^Tabelle1!$A8-1)/(Tabelle1!F$2*(1+Tabelle1!F$2)^Tabelle1!$A8),IF($B$1=Tabelle2!$A$4,(Tabelle1!F$2*(1+Tabelle1!F$2)^Tabelle1!$A8)/((1+Tabelle1!F$2)^Tabelle1!$A8-1)))))</f>
-        <v>5.0756920672674468</v>
-      </c>
-      <c r="G8" s="11">
+        <v>0.19701746811018833</v>
+      </c>
+      <c r="G8" s="8">
         <f>IF($B$1=Tabelle2!$A$1,(1+Tabelle1!G$2)^Tabelle1!$A8,IF($B$1=Tabelle2!$A$2,(1+Tabelle1!G$2)^(-Tabelle1!$A8),IF($B$1=Tabelle2!$A$3,((1+Tabelle1!G$2)^Tabelle1!$A8-1)/(Tabelle1!G$2*(1+Tabelle1!G$2)^Tabelle1!$A8),IF($B$1=Tabelle2!$A$4,(Tabelle1!G$2*(1+Tabelle1!G$2)^Tabelle1!$A8)/((1+Tabelle1!G$2)^Tabelle1!$A8-1)))))</f>
-        <v>4.9173243260053949</v>
-      </c>
-      <c r="H8" s="11">
+        <v>0.20336262847489528</v>
+      </c>
+      <c r="H8" s="8">
         <f>IF($B$1=Tabelle2!$A$1,(1+Tabelle1!H$2)^Tabelle1!$A8,IF($B$1=Tabelle2!$A$2,(1+Tabelle1!H$2)^(-Tabelle1!$A8),IF($B$1=Tabelle2!$A$3,((1+Tabelle1!H$2)^Tabelle1!$A8-1)/(Tabelle1!H$2*(1+Tabelle1!H$2)^Tabelle1!$A8),IF($B$1=Tabelle2!$A$4,(Tabelle1!H$2*(1+Tabelle1!H$2)^Tabelle1!$A8)/((1+Tabelle1!H$2)^Tabelle1!$A8-1)))))</f>
-        <v>4.7665396597641063</v>
-      </c>
-      <c r="I8" s="11">
+        <v>0.20979579975832816</v>
+      </c>
+      <c r="I8" s="8">
         <f>IF($B$1=Tabelle2!$A$1,(1+Tabelle1!I$2)^Tabelle1!$A8,IF($B$1=Tabelle2!$A$2,(1+Tabelle1!I$2)^(-Tabelle1!$A8),IF($B$1=Tabelle2!$A$3,((1+Tabelle1!I$2)^Tabelle1!$A8-1)/(Tabelle1!I$2*(1+Tabelle1!I$2)^Tabelle1!$A8),IF($B$1=Tabelle2!$A$4,(Tabelle1!I$2*(1+Tabelle1!I$2)^Tabelle1!$A8)/((1+Tabelle1!I$2)^Tabelle1!$A8-1)))))</f>
-        <v>4.6228796639611929</v>
-      </c>
-      <c r="J8" s="11">
+        <v>0.2163153862290097</v>
+      </c>
+      <c r="J8" s="8">
         <f>IF($B$1=Tabelle2!$A$1,(1+Tabelle1!J$2)^Tabelle1!$A8,IF($B$1=Tabelle2!$A$2,(1+Tabelle1!J$2)^(-Tabelle1!$A8),IF($B$1=Tabelle2!$A$3,((1+Tabelle1!J$2)^Tabelle1!$A8-1)/(Tabelle1!J$2*(1+Tabelle1!J$2)^Tabelle1!$A8),IF($B$1=Tabelle2!$A$4,(Tabelle1!J$2*(1+Tabelle1!J$2)^Tabelle1!$A8)/((1+Tabelle1!J$2)^Tabelle1!$A8-1)))))</f>
-        <v>4.485918590230936</v>
-      </c>
-      <c r="K8" s="11">
+        <v>0.22291978329203693</v>
+      </c>
+      <c r="K8" s="8">
         <f>IF($B$1=Tabelle2!$A$1,(1+Tabelle1!K$2)^Tabelle1!$A8,IF($B$1=Tabelle2!$A$2,(1+Tabelle1!K$2)^(-Tabelle1!$A8),IF($B$1=Tabelle2!$A$3,((1+Tabelle1!K$2)^Tabelle1!$A8-1)/(Tabelle1!K$2*(1+Tabelle1!K$2)^Tabelle1!$A8),IF($B$1=Tabelle2!$A$4,(Tabelle1!K$2*(1+Tabelle1!K$2)^Tabelle1!$A8)/((1+Tabelle1!K$2)^Tabelle1!$A8-1)))))</f>
-        <v>4.355260699462228</v>
-      </c>
-      <c r="L8" s="11">
+        <v>0.22960738036266726</v>
+      </c>
+      <c r="L8" s="8">
         <f>IF($B$1=Tabelle2!$A$1,(1+Tabelle1!L$2)^Tabelle1!$A8,IF($B$1=Tabelle2!$A$2,(1+Tabelle1!L$2)^(-Tabelle1!$A8),IF($B$1=Tabelle2!$A$3,((1+Tabelle1!L$2)^Tabelle1!$A8-1)/(Tabelle1!L$2*(1+Tabelle1!L$2)^Tabelle1!$A8),IF($B$1=Tabelle2!$A$4,(Tabelle1!L$2*(1+Tabelle1!L$2)^Tabelle1!$A8)/((1+Tabelle1!L$2)^Tabelle1!$A8-1)))))</f>
-        <v>4.2305378537382587</v>
-      </c>
-      <c r="M8" s="11">
+        <v>0.23637656358903947</v>
+      </c>
+      <c r="M8" s="8">
         <f>IF($B$1=Tabelle2!$A$1,(1+Tabelle1!M$2)^Tabelle1!$A8,IF($B$1=Tabelle2!$A$2,(1+Tabelle1!M$2)^(-Tabelle1!$A8),IF($B$1=Tabelle2!$A$3,((1+Tabelle1!M$2)^Tabelle1!$A8-1)/(Tabelle1!M$2*(1+Tabelle1!M$2)^Tabelle1!$A8),IF($B$1=Tabelle2!$A$4,(Tabelle1!M$2*(1+Tabelle1!M$2)^Tabelle1!$A8)/((1+Tabelle1!M$2)^Tabelle1!$A8-1)))))</f>
-        <v>4.1114073235223279</v>
+        <v>0.24322571842462917</v>
       </c>
     </row>
     <row r="9" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A9" s="6">
         <v>7</v>
       </c>
-      <c r="B9" s="11">
+      <c r="B9" s="8">
         <f>IF($B$1=Tabelle2!$A$1,(1+Tabelle1!B$2)^Tabelle1!$A9,IF($B$1=Tabelle2!$A$2,(1+Tabelle1!B$2)^(-Tabelle1!$A9),IF($B$1=Tabelle2!$A$3,((1+Tabelle1!B$2)^Tabelle1!$A9-1)/(Tabelle1!B$2*(1+Tabelle1!B$2)^Tabelle1!$A9),IF($B$1=Tabelle2!$A$4,(Tabelle1!B$2*(1+Tabelle1!B$2)^Tabelle1!$A9)/((1+Tabelle1!B$2)^Tabelle1!$A9-1)))))</f>
-        <v>6.7281945292864478</v>
-      </c>
-      <c r="C9" s="11">
+        <v>0.14862828291411692</v>
+      </c>
+      <c r="C9" s="8">
         <f>IF($B$1=Tabelle2!$A$1,(1+Tabelle1!C$2)^Tabelle1!$A9,IF($B$1=Tabelle2!$A$2,(1+Tabelle1!C$2)^(-Tabelle1!$A9),IF($B$1=Tabelle2!$A$3,((1+Tabelle1!C$2)^Tabelle1!$A9-1)/(Tabelle1!C$2*(1+Tabelle1!C$2)^Tabelle1!$A9),IF($B$1=Tabelle2!$A$4,(Tabelle1!C$2*(1+Tabelle1!C$2)^Tabelle1!$A9)/((1+Tabelle1!C$2)^Tabelle1!$A9-1)))))</f>
-        <v>6.4719910693043046</v>
-      </c>
-      <c r="D9" s="11">
+        <v>0.1545119561030997</v>
+      </c>
+      <c r="D9" s="8">
         <f>IF($B$1=Tabelle2!$A$1,(1+Tabelle1!D$2)^Tabelle1!$A9,IF($B$1=Tabelle2!$A$2,(1+Tabelle1!D$2)^(-Tabelle1!$A9),IF($B$1=Tabelle2!$A$3,((1+Tabelle1!D$2)^Tabelle1!$A9-1)/(Tabelle1!D$2*(1+Tabelle1!D$2)^Tabelle1!$A9),IF($B$1=Tabelle2!$A$4,(Tabelle1!D$2*(1+Tabelle1!D$2)^Tabelle1!$A9)/((1+Tabelle1!D$2)^Tabelle1!$A9-1)))))</f>
-        <v>6.2302829552215409</v>
-      </c>
-      <c r="E9" s="11">
+        <v>0.16050635375427202</v>
+      </c>
+      <c r="E9" s="8">
         <f>IF($B$1=Tabelle2!$A$1,(1+Tabelle1!E$2)^Tabelle1!$A9,IF($B$1=Tabelle2!$A$2,(1+Tabelle1!E$2)^(-Tabelle1!$A9),IF($B$1=Tabelle2!$A$3,((1+Tabelle1!E$2)^Tabelle1!$A9-1)/(Tabelle1!E$2*(1+Tabelle1!E$2)^Tabelle1!$A9),IF($B$1=Tabelle2!$A$4,(Tabelle1!E$2*(1+Tabelle1!E$2)^Tabelle1!$A9)/((1+Tabelle1!E$2)^Tabelle1!$A9-1)))))</f>
-        <v>6.0020546699484187</v>
-      </c>
-      <c r="F9" s="11">
+        <v>0.16660961203950414</v>
+      </c>
+      <c r="F9" s="8">
         <f>IF($B$1=Tabelle2!$A$1,(1+Tabelle1!F$2)^Tabelle1!$A9,IF($B$1=Tabelle2!$A$2,(1+Tabelle1!F$2)^(-Tabelle1!$A9),IF($B$1=Tabelle2!$A$3,((1+Tabelle1!F$2)^Tabelle1!$A9-1)/(Tabelle1!F$2*(1+Tabelle1!F$2)^Tabelle1!$A9),IF($B$1=Tabelle2!$A$4,(Tabelle1!F$2*(1+Tabelle1!F$2)^Tabelle1!$A9)/((1+Tabelle1!F$2)^Tabelle1!$A9-1)))))</f>
-        <v>5.7863733973975711</v>
-      </c>
-      <c r="G9" s="11">
+        <v>0.17281981844617067</v>
+      </c>
+      <c r="G9" s="8">
         <f>IF($B$1=Tabelle2!$A$1,(1+Tabelle1!G$2)^Tabelle1!$A9,IF($B$1=Tabelle2!$A$2,(1+Tabelle1!G$2)^(-Tabelle1!$A9),IF($B$1=Tabelle2!$A$3,((1+Tabelle1!G$2)^Tabelle1!$A9-1)/(Tabelle1!G$2*(1+Tabelle1!G$2)^Tabelle1!$A9),IF($B$1=Tabelle2!$A$4,(Tabelle1!G$2*(1+Tabelle1!G$2)^Tabelle1!$A9)/((1+Tabelle1!G$2)^Tabelle1!$A9-1)))))</f>
-        <v>5.5823814396277331</v>
-      </c>
-      <c r="H9" s="11">
+        <v>0.17913501805901069</v>
+      </c>
+      <c r="H9" s="8">
         <f>IF($B$1=Tabelle2!$A$1,(1+Tabelle1!H$2)^Tabelle1!$A9,IF($B$1=Tabelle2!$A$2,(1+Tabelle1!H$2)^(-Tabelle1!$A9),IF($B$1=Tabelle2!$A$3,((1+Tabelle1!H$2)^Tabelle1!$A9-1)/(Tabelle1!H$2*(1+Tabelle1!H$2)^Tabelle1!$A9),IF($B$1=Tabelle2!$A$4,(Tabelle1!H$2*(1+Tabelle1!H$2)^Tabelle1!$A9)/((1+Tabelle1!H$2)^Tabelle1!$A9-1)))))</f>
-        <v>5.3892894016486981</v>
-      </c>
-      <c r="I9" s="11">
+        <v>0.18555321963115931</v>
+      </c>
+      <c r="I9" s="8">
         <f>IF($B$1=Tabelle2!$A$1,(1+Tabelle1!I$2)^Tabelle1!$A9,IF($B$1=Tabelle2!$A$2,(1+Tabelle1!I$2)^(-Tabelle1!$A9),IF($B$1=Tabelle2!$A$3,((1+Tabelle1!I$2)^Tabelle1!$A9-1)/(Tabelle1!I$2*(1+Tabelle1!I$2)^Tabelle1!$A9),IF($B$1=Tabelle2!$A$4,(Tabelle1!I$2*(1+Tabelle1!I$2)^Tabelle1!$A9)/((1+Tabelle1!I$2)^Tabelle1!$A9-1)))))</f>
-        <v>5.2063700592233264</v>
-      </c>
-      <c r="J9" s="11">
+        <v>0.19207240142841048</v>
+      </c>
+      <c r="J9" s="8">
         <f>IF($B$1=Tabelle2!$A$1,(1+Tabelle1!J$2)^Tabelle1!$A9,IF($B$1=Tabelle2!$A$2,(1+Tabelle1!J$2)^(-Tabelle1!$A9),IF($B$1=Tabelle2!$A$3,((1+Tabelle1!J$2)^Tabelle1!$A9-1)/(Tabelle1!J$2*(1+Tabelle1!J$2)^Tabelle1!$A9),IF($B$1=Tabelle2!$A$4,(Tabelle1!J$2*(1+Tabelle1!J$2)^Tabelle1!$A9)/((1+Tabelle1!J$2)^Tabelle1!$A9-1)))))</f>
-        <v>5.0329528350742532</v>
-      </c>
-      <c r="K9" s="11">
+        <v>0.1986905168335929</v>
+      </c>
+      <c r="K9" s="8">
         <f>IF($B$1=Tabelle2!$A$1,(1+Tabelle1!K$2)^Tabelle1!$A9,IF($B$1=Tabelle2!$A$2,(1+Tabelle1!K$2)^(-Tabelle1!$A9),IF($B$1=Tabelle2!$A$3,((1+Tabelle1!K$2)^Tabelle1!$A9-1)/(Tabelle1!K$2*(1+Tabelle1!K$2)^Tabelle1!$A9),IF($B$1=Tabelle2!$A$4,(Tabelle1!K$2*(1+Tabelle1!K$2)^Tabelle1!$A9)/((1+Tabelle1!K$2)^Tabelle1!$A9-1)))))</f>
-        <v>4.8684188176929348</v>
-      </c>
-      <c r="L9" s="11">
+        <v>0.20540549970059557</v>
+      </c>
+      <c r="L9" s="8">
         <f>IF($B$1=Tabelle2!$A$1,(1+Tabelle1!L$2)^Tabelle1!$A9,IF($B$1=Tabelle2!$A$2,(1+Tabelle1!L$2)^(-Tabelle1!$A9),IF($B$1=Tabelle2!$A$3,((1+Tabelle1!L$2)^Tabelle1!$A9-1)/(Tabelle1!L$2*(1+Tabelle1!L$2)^Tabelle1!$A9),IF($B$1=Tabelle2!$A$4,(Tabelle1!L$2*(1+Tabelle1!L$2)^Tabelle1!$A9)/((1+Tabelle1!L$2)^Tabelle1!$A9-1)))))</f>
-        <v>4.7121962646290623</v>
-      </c>
-      <c r="M9" s="11">
+        <v>0.21221526945009764</v>
+      </c>
+      <c r="M9" s="8">
         <f>IF($B$1=Tabelle2!$A$1,(1+Tabelle1!M$2)^Tabelle1!$A9,IF($B$1=Tabelle2!$A$2,(1+Tabelle1!M$2)^(-Tabelle1!$A9),IF($B$1=Tabelle2!$A$3,((1+Tabelle1!M$2)^Tabelle1!$A9-1)/(Tabelle1!M$2*(1+Tabelle1!M$2)^Tabelle1!$A9),IF($B$1=Tabelle2!$A$4,(Tabelle1!M$2*(1+Tabelle1!M$2)^Tabelle1!$A9)/((1+Tabelle1!M$2)^Tabelle1!$A9-1)))))</f>
-        <v>4.5637565388592209</v>
+        <v>0.21911773590139078</v>
       </c>
     </row>
     <row r="10" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A10" s="6">
         <v>8</v>
       </c>
-      <c r="B10" s="11">
+      <c r="B10" s="8">
         <f>IF($B$1=Tabelle2!$A$1,(1+Tabelle1!B$2)^Tabelle1!$A10,IF($B$1=Tabelle2!$A$2,(1+Tabelle1!B$2)^(-Tabelle1!$A10),IF($B$1=Tabelle2!$A$3,((1+Tabelle1!B$2)^Tabelle1!$A10-1)/(Tabelle1!B$2*(1+Tabelle1!B$2)^Tabelle1!$A10),IF($B$1=Tabelle2!$A$4,(Tabelle1!B$2*(1+Tabelle1!B$2)^Tabelle1!$A10)/((1+Tabelle1!B$2)^Tabelle1!$A10-1)))))</f>
-        <v>7.6516777517687862</v>
-      </c>
-      <c r="C10" s="11">
+        <v>0.13069029204331517</v>
+      </c>
+      <c r="C10" s="8">
         <f>IF($B$1=Tabelle2!$A$1,(1+Tabelle1!C$2)^Tabelle1!$A10,IF($B$1=Tabelle2!$A$2,(1+Tabelle1!C$2)^(-Tabelle1!$A10),IF($B$1=Tabelle2!$A$3,((1+Tabelle1!C$2)^Tabelle1!$A10-1)/(Tabelle1!C$2*(1+Tabelle1!C$2)^Tabelle1!$A10),IF($B$1=Tabelle2!$A$4,(Tabelle1!C$2*(1+Tabelle1!C$2)^Tabelle1!$A10)/((1+Tabelle1!C$2)^Tabelle1!$A10-1)))))</f>
-        <v>7.3254814404944195</v>
-      </c>
-      <c r="D10" s="11">
+        <v>0.13650979913376274</v>
+      </c>
+      <c r="D10" s="8">
         <f>IF($B$1=Tabelle2!$A$1,(1+Tabelle1!D$2)^Tabelle1!$A10,IF($B$1=Tabelle2!$A$2,(1+Tabelle1!D$2)^(-Tabelle1!$A10),IF($B$1=Tabelle2!$A$3,((1+Tabelle1!D$2)^Tabelle1!$A10-1)/(Tabelle1!D$2*(1+Tabelle1!D$2)^Tabelle1!$A10),IF($B$1=Tabelle2!$A$4,(Tabelle1!D$2*(1+Tabelle1!D$2)^Tabelle1!$A10)/((1+Tabelle1!D$2)^Tabelle1!$A10-1)))))</f>
-        <v>7.0196921895354745</v>
-      </c>
-      <c r="E10" s="11">
+        <v>0.14245638882723924</v>
+      </c>
+      <c r="E10" s="8">
         <f>IF($B$1=Tabelle2!$A$1,(1+Tabelle1!E$2)^Tabelle1!$A10,IF($B$1=Tabelle2!$A$2,(1+Tabelle1!E$2)^(-Tabelle1!$A10),IF($B$1=Tabelle2!$A$3,((1+Tabelle1!E$2)^Tabelle1!$A10-1)/(Tabelle1!E$2*(1+Tabelle1!E$2)^Tabelle1!$A10),IF($B$1=Tabelle2!$A$4,(Tabelle1!E$2*(1+Tabelle1!E$2)^Tabelle1!$A10)/((1+Tabelle1!E$2)^Tabelle1!$A10-1)))))</f>
-        <v>6.7327448749504057</v>
-      </c>
-      <c r="F10" s="11">
+        <v>0.14852783204671277</v>
+      </c>
+      <c r="F10" s="8">
         <f>IF($B$1=Tabelle2!$A$1,(1+Tabelle1!F$2)^Tabelle1!$A10,IF($B$1=Tabelle2!$A$2,(1+Tabelle1!F$2)^(-Tabelle1!$A10),IF($B$1=Tabelle2!$A$3,((1+Tabelle1!F$2)^Tabelle1!$A10-1)/(Tabelle1!F$2*(1+Tabelle1!F$2)^Tabelle1!$A10),IF($B$1=Tabelle2!$A$4,(Tabelle1!F$2*(1+Tabelle1!F$2)^Tabelle1!$A10)/((1+Tabelle1!F$2)^Tabelle1!$A10-1)))))</f>
-        <v>6.4632127594262556</v>
-      </c>
-      <c r="G10" s="11">
+        <v>0.15472181362768117</v>
+      </c>
+      <c r="G10" s="8">
         <f>IF($B$1=Tabelle2!$A$1,(1+Tabelle1!G$2)^Tabelle1!$A10,IF($B$1=Tabelle2!$A$2,(1+Tabelle1!G$2)^(-Tabelle1!$A10),IF($B$1=Tabelle2!$A$3,((1+Tabelle1!G$2)^Tabelle1!$A10-1)/(Tabelle1!G$2*(1+Tabelle1!G$2)^Tabelle1!$A10),IF($B$1=Tabelle2!$A$4,(Tabelle1!G$2*(1+Tabelle1!G$2)^Tabelle1!$A10)/((1+Tabelle1!G$2)^Tabelle1!$A10-1)))))</f>
-        <v>6.2097938109695585</v>
-      </c>
-      <c r="H10" s="11">
+        <v>0.16103594264812895</v>
+      </c>
+      <c r="H10" s="8">
         <f>IF($B$1=Tabelle2!$A$1,(1+Tabelle1!H$2)^Tabelle1!$A10,IF($B$1=Tabelle2!$A$2,(1+Tabelle1!H$2)^(-Tabelle1!$A10),IF($B$1=Tabelle2!$A$3,((1+Tabelle1!H$2)^Tabelle1!$A10-1)/(Tabelle1!H$2*(1+Tabelle1!H$2)^Tabelle1!$A10),IF($B$1=Tabelle2!$A$4,(Tabelle1!H$2*(1+Tabelle1!H$2)^Tabelle1!$A10)/((1+Tabelle1!H$2)^Tabelle1!$A10-1)))))</f>
-        <v>5.9712985062137367</v>
-      </c>
-      <c r="I10" s="11">
+        <v>0.16746776249075465</v>
+      </c>
+      <c r="I10" s="8">
         <f>IF($B$1=Tabelle2!$A$1,(1+Tabelle1!I$2)^Tabelle1!$A10,IF($B$1=Tabelle2!$A$2,(1+Tabelle1!I$2)^(-Tabelle1!$A10),IF($B$1=Tabelle2!$A$3,((1+Tabelle1!I$2)^Tabelle1!$A10-1)/(Tabelle1!I$2*(1+Tabelle1!I$2)^Tabelle1!$A10),IF($B$1=Tabelle2!$A$4,(Tabelle1!I$2*(1+Tabelle1!I$2)^Tabelle1!$A10)/((1+Tabelle1!I$2)^Tabelle1!$A10-1)))))</f>
-        <v>5.7466389437253023</v>
-      </c>
-      <c r="J10" s="11">
+        <v>0.17401476059182211</v>
+      </c>
+      <c r="J10" s="8">
         <f>IF($B$1=Tabelle2!$A$1,(1+Tabelle1!J$2)^Tabelle1!$A10,IF($B$1=Tabelle2!$A$2,(1+Tabelle1!J$2)^(-Tabelle1!$A10),IF($B$1=Tabelle2!$A$3,((1+Tabelle1!J$2)^Tabelle1!$A10-1)/(Tabelle1!J$2*(1+Tabelle1!J$2)^Tabelle1!$A10),IF($B$1=Tabelle2!$A$4,(Tabelle1!J$2*(1+Tabelle1!J$2)^Tabelle1!$A10)/((1+Tabelle1!J$2)^Tabelle1!$A10-1)))))</f>
-        <v>5.5348191147470214</v>
-      </c>
-      <c r="K10" s="11">
+        <v>0.18067437783749629</v>
+      </c>
+      <c r="K10" s="8">
         <f>IF($B$1=Tabelle2!$A$1,(1+Tabelle1!K$2)^Tabelle1!$A10,IF($B$1=Tabelle2!$A$2,(1+Tabelle1!K$2)^(-Tabelle1!$A10),IF($B$1=Tabelle2!$A$3,((1+Tabelle1!K$2)^Tabelle1!$A10-1)/(Tabelle1!K$2*(1+Tabelle1!K$2)^Tabelle1!$A10),IF($B$1=Tabelle2!$A$4,(Tabelle1!K$2*(1+Tabelle1!K$2)^Tabelle1!$A10)/((1+Tabelle1!K$2)^Tabelle1!$A10-1)))))</f>
-        <v>5.3349261979026679</v>
-      </c>
-      <c r="L10" s="11">
+        <v>0.18744401757481335</v>
+      </c>
+      <c r="L10" s="8">
         <f>IF($B$1=Tabelle2!$A$1,(1+Tabelle1!L$2)^Tabelle1!$A10,IF($B$1=Tabelle2!$A$2,(1+Tabelle1!L$2)^(-Tabelle1!$A10),IF($B$1=Tabelle2!$A$3,((1+Tabelle1!L$2)^Tabelle1!$A10-1)/(Tabelle1!L$2*(1+Tabelle1!L$2)^Tabelle1!$A10),IF($B$1=Tabelle2!$A$4,(Tabelle1!L$2*(1+Tabelle1!L$2)^Tabelle1!$A10)/((1+Tabelle1!L$2)^Tabelle1!$A10-1)))))</f>
-        <v>5.1461227609270841</v>
-      </c>
-      <c r="M10" s="11">
+        <v>0.19432105421050003</v>
+      </c>
+      <c r="M10" s="8">
         <f>IF($B$1=Tabelle2!$A$1,(1+Tabelle1!M$2)^Tabelle1!$A10,IF($B$1=Tabelle2!$A$2,(1+Tabelle1!M$2)^(-Tabelle1!$A10),IF($B$1=Tabelle2!$A$3,((1+Tabelle1!M$2)^Tabelle1!$A10-1)/(Tabelle1!M$2*(1+Tabelle1!M$2)^Tabelle1!$A10),IF($B$1=Tabelle2!$A$4,(Tabelle1!M$2*(1+Tabelle1!M$2)^Tabelle1!$A10)/((1+Tabelle1!M$2)^Tabelle1!$A10-1)))))</f>
-        <v>4.967639766838591</v>
+        <v>0.20130284137660018</v>
       </c>
     </row>
     <row r="11" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A11" s="6">
         <v>9</v>
       </c>
-      <c r="B11" s="11">
+      <c r="B11" s="8">
         <f>IF($B$1=Tabelle2!$A$1,(1+Tabelle1!B$2)^Tabelle1!$A11,IF($B$1=Tabelle2!$A$2,(1+Tabelle1!B$2)^(-Tabelle1!$A11),IF($B$1=Tabelle2!$A$3,((1+Tabelle1!B$2)^Tabelle1!$A11-1)/(Tabelle1!B$2*(1+Tabelle1!B$2)^Tabelle1!$A11),IF($B$1=Tabelle2!$A$4,(Tabelle1!B$2*(1+Tabelle1!B$2)^Tabelle1!$A11)/((1+Tabelle1!B$2)^Tabelle1!$A11-1)))))</f>
-        <v>8.5660175760087043</v>
-      </c>
-      <c r="C11" s="11">
+        <v>0.11674036284968087</v>
+      </c>
+      <c r="C11" s="8">
         <f>IF($B$1=Tabelle2!$A$1,(1+Tabelle1!C$2)^Tabelle1!$A11,IF($B$1=Tabelle2!$A$2,(1+Tabelle1!C$2)^(-Tabelle1!$A11),IF($B$1=Tabelle2!$A$3,((1+Tabelle1!C$2)^Tabelle1!$A11-1)/(Tabelle1!C$2*(1+Tabelle1!C$2)^Tabelle1!$A11),IF($B$1=Tabelle2!$A$4,(Tabelle1!C$2*(1+Tabelle1!C$2)^Tabelle1!$A11)/((1+Tabelle1!C$2)^Tabelle1!$A11-1)))))</f>
-        <v>8.1622367063670787</v>
-      </c>
-      <c r="D11" s="11">
+        <v>0.12251543737024126</v>
+      </c>
+      <c r="D11" s="8">
         <f>IF($B$1=Tabelle2!$A$1,(1+Tabelle1!D$2)^Tabelle1!$A11,IF($B$1=Tabelle2!$A$2,(1+Tabelle1!D$2)^(-Tabelle1!$A11),IF($B$1=Tabelle2!$A$3,((1+Tabelle1!D$2)^Tabelle1!$A11-1)/(Tabelle1!D$2*(1+Tabelle1!D$2)^Tabelle1!$A11),IF($B$1=Tabelle2!$A$4,(Tabelle1!D$2*(1+Tabelle1!D$2)^Tabelle1!$A11)/((1+Tabelle1!D$2)^Tabelle1!$A11-1)))))</f>
-        <v>7.7861089218791015</v>
-      </c>
-      <c r="E11" s="11">
+        <v>0.12843385701810342</v>
+      </c>
+      <c r="E11" s="8">
         <f>IF($B$1=Tabelle2!$A$1,(1+Tabelle1!E$2)^Tabelle1!$A11,IF($B$1=Tabelle2!$A$2,(1+Tabelle1!E$2)^(-Tabelle1!$A11),IF($B$1=Tabelle2!$A$3,((1+Tabelle1!E$2)^Tabelle1!$A11-1)/(Tabelle1!E$2*(1+Tabelle1!E$2)^Tabelle1!$A11),IF($B$1=Tabelle2!$A$4,(Tabelle1!E$2*(1+Tabelle1!E$2)^Tabelle1!$A11)/((1+Tabelle1!E$2)^Tabelle1!$A11-1)))))</f>
-        <v>7.4353316105292375</v>
-      </c>
-      <c r="F11" s="11">
+        <v>0.13449299269771522</v>
+      </c>
+      <c r="F11" s="8">
         <f>IF($B$1=Tabelle2!$A$1,(1+Tabelle1!F$2)^Tabelle1!$A11,IF($B$1=Tabelle2!$A$2,(1+Tabelle1!F$2)^(-Tabelle1!$A11),IF($B$1=Tabelle2!$A$3,((1+Tabelle1!F$2)^Tabelle1!$A11-1)/(Tabelle1!F$2*(1+Tabelle1!F$2)^Tabelle1!$A11),IF($B$1=Tabelle2!$A$4,(Tabelle1!F$2*(1+Tabelle1!F$2)^Tabelle1!$A11)/((1+Tabelle1!F$2)^Tabelle1!$A11-1)))))</f>
-        <v>7.107821675644054</v>
-      </c>
-      <c r="G11" s="11">
+        <v>0.14069007997578778</v>
+      </c>
+      <c r="G11" s="8">
         <f>IF($B$1=Tabelle2!$A$1,(1+Tabelle1!G$2)^Tabelle1!$A11,IF($B$1=Tabelle2!$A$2,(1+Tabelle1!G$2)^(-Tabelle1!$A11),IF($B$1=Tabelle2!$A$3,((1+Tabelle1!G$2)^Tabelle1!$A11-1)/(Tabelle1!G$2*(1+Tabelle1!G$2)^Tabelle1!$A11),IF($B$1=Tabelle2!$A$4,(Tabelle1!G$2*(1+Tabelle1!G$2)^Tabelle1!$A11)/((1+Tabelle1!G$2)^Tabelle1!$A11-1)))))</f>
-        <v>6.8016922744995831</v>
-      </c>
-      <c r="H11" s="11">
+        <v>0.14702223500306361</v>
+      </c>
+      <c r="H11" s="8">
         <f>IF($B$1=Tabelle2!$A$1,(1+Tabelle1!H$2)^Tabelle1!$A11,IF($B$1=Tabelle2!$A$2,(1+Tabelle1!H$2)^(-Tabelle1!$A11),IF($B$1=Tabelle2!$A$3,((1+Tabelle1!H$2)^Tabelle1!$A11-1)/(Tabelle1!H$2*(1+Tabelle1!H$2)^Tabelle1!$A11),IF($B$1=Tabelle2!$A$4,(Tabelle1!H$2*(1+Tabelle1!H$2)^Tabelle1!$A11)/((1+Tabelle1!H$2)^Tabelle1!$A11-1)))))</f>
-        <v>6.5152322487978847</v>
-      </c>
-      <c r="I11" s="11">
+        <v>0.15348647013842193</v>
+      </c>
+      <c r="I11" s="8">
         <f>IF($B$1=Tabelle2!$A$1,(1+Tabelle1!I$2)^Tabelle1!$A11,IF($B$1=Tabelle2!$A$2,(1+Tabelle1!I$2)^(-Tabelle1!$A11),IF($B$1=Tabelle2!$A$3,((1+Tabelle1!I$2)^Tabelle1!$A11-1)/(Tabelle1!I$2*(1+Tabelle1!I$2)^Tabelle1!$A11),IF($B$1=Tabelle2!$A$4,(Tabelle1!I$2*(1+Tabelle1!I$2)^Tabelle1!$A11)/((1+Tabelle1!I$2)^Tabelle1!$A11-1)))))</f>
-        <v>6.2468879108567625</v>
-      </c>
-      <c r="J11" s="11">
+        <v>0.16007970917199468</v>
+      </c>
+      <c r="J11" s="8">
         <f>IF($B$1=Tabelle2!$A$1,(1+Tabelle1!J$2)^Tabelle1!$A11,IF($B$1=Tabelle2!$A$2,(1+Tabelle1!J$2)^(-Tabelle1!$A11),IF($B$1=Tabelle2!$A$3,((1+Tabelle1!J$2)^Tabelle1!$A11-1)/(Tabelle1!J$2*(1+Tabelle1!J$2)^Tabelle1!$A11),IF($B$1=Tabelle2!$A$4,(Tabelle1!J$2*(1+Tabelle1!J$2)^Tabelle1!$A11)/((1+Tabelle1!J$2)^Tabelle1!$A11-1)))))</f>
-        <v>5.9952468942633228</v>
-      </c>
-      <c r="K11" s="11">
+        <v>0.1667988020571548</v>
+      </c>
+      <c r="K11" s="8">
         <f>IF($B$1=Tabelle2!$A$1,(1+Tabelle1!K$2)^Tabelle1!$A11,IF($B$1=Tabelle2!$A$2,(1+Tabelle1!K$2)^(-Tabelle1!$A11),IF($B$1=Tabelle2!$A$3,((1+Tabelle1!K$2)^Tabelle1!$A11-1)/(Tabelle1!K$2*(1+Tabelle1!K$2)^Tabelle1!$A11),IF($B$1=Tabelle2!$A$4,(Tabelle1!K$2*(1+Tabelle1!K$2)^Tabelle1!$A11)/((1+Tabelle1!K$2)^Tabelle1!$A11-1)))))</f>
-        <v>5.7590238162751533</v>
-      </c>
-      <c r="L11" s="11">
+        <v>0.1736405390743434</v>
+      </c>
+      <c r="L11" s="8">
         <f>IF($B$1=Tabelle2!$A$1,(1+Tabelle1!L$2)^Tabelle1!$A11,IF($B$1=Tabelle2!$A$2,(1+Tabelle1!L$2)^(-Tabelle1!$A11),IF($B$1=Tabelle2!$A$3,((1+Tabelle1!L$2)^Tabelle1!$A11-1)/(Tabelle1!L$2*(1+Tabelle1!L$2)^Tabelle1!$A11),IF($B$1=Tabelle2!$A$4,(Tabelle1!L$2*(1+Tabelle1!L$2)^Tabelle1!$A11)/((1+Tabelle1!L$2)^Tabelle1!$A11-1)))))</f>
-        <v>5.5370475323667421</v>
-      </c>
-      <c r="M11" s="11">
+        <v>0.18060166436255287</v>
+      </c>
+      <c r="M11" s="8">
         <f>IF($B$1=Tabelle2!$A$1,(1+Tabelle1!M$2)^Tabelle1!$A11,IF($B$1=Tabelle2!$A$2,(1+Tabelle1!M$2)^(-Tabelle1!$A11),IF($B$1=Tabelle2!$A$3,((1+Tabelle1!M$2)^Tabelle1!$A11-1)/(Tabelle1!M$2*(1+Tabelle1!M$2)^Tabelle1!$A11),IF($B$1=Tabelle2!$A$4,(Tabelle1!M$2*(1+Tabelle1!M$2)^Tabelle1!$A11)/((1+Tabelle1!M$2)^Tabelle1!$A11-1)))))</f>
-        <v>5.3282497918201699</v>
+        <v>0.18767888876666056</v>
       </c>
     </row>
     <row r="12" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A12" s="6">
         <v>10</v>
       </c>
-      <c r="B12" s="11">
+      <c r="B12" s="8">
         <f>IF($B$1=Tabelle2!$A$1,(1+Tabelle1!B$2)^Tabelle1!$A12,IF($B$1=Tabelle2!$A$2,(1+Tabelle1!B$2)^(-Tabelle1!$A12),IF($B$1=Tabelle2!$A$3,((1+Tabelle1!B$2)^Tabelle1!$A12-1)/(Tabelle1!B$2*(1+Tabelle1!B$2)^Tabelle1!$A12),IF($B$1=Tabelle2!$A$4,(Tabelle1!B$2*(1+Tabelle1!B$2)^Tabelle1!$A12)/((1+Tabelle1!B$2)^Tabelle1!$A12-1)))))</f>
-        <v>9.4713045307016905</v>
-      </c>
-      <c r="C12" s="11">
+        <v>0.10558207655117115</v>
+      </c>
+      <c r="C12" s="8">
         <f>IF($B$1=Tabelle2!$A$1,(1+Tabelle1!C$2)^Tabelle1!$A12,IF($B$1=Tabelle2!$A$2,(1+Tabelle1!C$2)^(-Tabelle1!$A12),IF($B$1=Tabelle2!$A$3,((1+Tabelle1!C$2)^Tabelle1!$A12-1)/(Tabelle1!C$2*(1+Tabelle1!C$2)^Tabelle1!$A12),IF($B$1=Tabelle2!$A$4,(Tabelle1!C$2*(1+Tabelle1!C$2)^Tabelle1!$A12)/((1+Tabelle1!C$2)^Tabelle1!$A12-1)))))</f>
-        <v>8.9825850062422354</v>
-      </c>
-      <c r="D12" s="11">
+        <v>0.11132652786531647</v>
+      </c>
+      <c r="D12" s="8">
         <f>IF($B$1=Tabelle2!$A$1,(1+Tabelle1!D$2)^Tabelle1!$A12,IF($B$1=Tabelle2!$A$2,(1+Tabelle1!D$2)^(-Tabelle1!$A12),IF($B$1=Tabelle2!$A$3,((1+Tabelle1!D$2)^Tabelle1!$A12-1)/(Tabelle1!D$2*(1+Tabelle1!D$2)^Tabelle1!$A12),IF($B$1=Tabelle2!$A$4,(Tabelle1!D$2*(1+Tabelle1!D$2)^Tabelle1!$A12)/((1+Tabelle1!D$2)^Tabelle1!$A12-1)))))</f>
-        <v>8.5302028367758282</v>
-      </c>
-      <c r="E12" s="11">
+        <v>0.11723050660515963</v>
+      </c>
+      <c r="E12" s="8">
         <f>IF($B$1=Tabelle2!$A$1,(1+Tabelle1!E$2)^Tabelle1!$A12,IF($B$1=Tabelle2!$A$2,(1+Tabelle1!E$2)^(-Tabelle1!$A12),IF($B$1=Tabelle2!$A$3,((1+Tabelle1!E$2)^Tabelle1!$A12-1)/(Tabelle1!E$2*(1+Tabelle1!E$2)^Tabelle1!$A12),IF($B$1=Tabelle2!$A$4,(Tabelle1!E$2*(1+Tabelle1!E$2)^Tabelle1!$A12)/((1+Tabelle1!E$2)^Tabelle1!$A12-1)))))</f>
-        <v>8.1108957793550349</v>
-      </c>
-      <c r="F12" s="11">
+        <v>0.1232909443301364</v>
+      </c>
+      <c r="F12" s="8">
         <f>IF($B$1=Tabelle2!$A$1,(1+Tabelle1!F$2)^Tabelle1!$A12,IF($B$1=Tabelle2!$A$2,(1+Tabelle1!F$2)^(-Tabelle1!$A12),IF($B$1=Tabelle2!$A$3,((1+Tabelle1!F$2)^Tabelle1!$A12-1)/(Tabelle1!F$2*(1+Tabelle1!F$2)^Tabelle1!$A12),IF($B$1=Tabelle2!$A$4,(Tabelle1!F$2*(1+Tabelle1!F$2)^Tabelle1!$A12)/((1+Tabelle1!F$2)^Tabelle1!$A12-1)))))</f>
-        <v>7.7217349291848123</v>
-      </c>
-      <c r="G12" s="11">
+        <v>0.1295045749654567</v>
+      </c>
+      <c r="G12" s="8">
         <f>IF($B$1=Tabelle2!$A$1,(1+Tabelle1!G$2)^Tabelle1!$A12,IF($B$1=Tabelle2!$A$2,(1+Tabelle1!G$2)^(-Tabelle1!$A12),IF($B$1=Tabelle2!$A$3,((1+Tabelle1!G$2)^Tabelle1!$A12-1)/(Tabelle1!G$2*(1+Tabelle1!G$2)^Tabelle1!$A12),IF($B$1=Tabelle2!$A$4,(Tabelle1!G$2*(1+Tabelle1!G$2)^Tabelle1!$A12)/((1+Tabelle1!G$2)^Tabelle1!$A12-1)))))</f>
-        <v>7.3600870514147028</v>
-      </c>
-      <c r="H12" s="11">
+        <v>0.13586795822038372</v>
+      </c>
+      <c r="H12" s="8">
         <f>IF($B$1=Tabelle2!$A$1,(1+Tabelle1!H$2)^Tabelle1!$A12,IF($B$1=Tabelle2!$A$2,(1+Tabelle1!H$2)^(-Tabelle1!$A12),IF($B$1=Tabelle2!$A$3,((1+Tabelle1!H$2)^Tabelle1!$A12-1)/(Tabelle1!H$2*(1+Tabelle1!H$2)^Tabelle1!$A12),IF($B$1=Tabelle2!$A$4,(Tabelle1!H$2*(1+Tabelle1!H$2)^Tabelle1!$A12)/((1+Tabelle1!H$2)^Tabelle1!$A12-1)))))</f>
-        <v>7.0235815409326028</v>
-      </c>
-      <c r="I12" s="11">
+        <v>0.14237750272736471</v>
+      </c>
+      <c r="I12" s="8">
         <f>IF($B$1=Tabelle2!$A$1,(1+Tabelle1!I$2)^Tabelle1!$A12,IF($B$1=Tabelle2!$A$2,(1+Tabelle1!I$2)^(-Tabelle1!$A12),IF($B$1=Tabelle2!$A$3,((1+Tabelle1!I$2)^Tabelle1!$A12-1)/(Tabelle1!I$2*(1+Tabelle1!I$2)^Tabelle1!$A12),IF($B$1=Tabelle2!$A$4,(Tabelle1!I$2*(1+Tabelle1!I$2)^Tabelle1!$A12)/((1+Tabelle1!I$2)^Tabelle1!$A12-1)))))</f>
-        <v>6.7100813989414467</v>
-      </c>
-      <c r="J12" s="11">
+        <v>0.14902948869707539</v>
+      </c>
+      <c r="J12" s="8">
         <f>IF($B$1=Tabelle2!$A$1,(1+Tabelle1!J$2)^Tabelle1!$A12,IF($B$1=Tabelle2!$A$2,(1+Tabelle1!J$2)^(-Tabelle1!$A12),IF($B$1=Tabelle2!$A$3,((1+Tabelle1!J$2)^Tabelle1!$A12-1)/(Tabelle1!J$2*(1+Tabelle1!J$2)^Tabelle1!$A12),IF($B$1=Tabelle2!$A$4,(Tabelle1!J$2*(1+Tabelle1!J$2)^Tabelle1!$A12)/((1+Tabelle1!J$2)^Tabelle1!$A12-1)))))</f>
-        <v>6.4176577011590119</v>
-      </c>
-      <c r="K12" s="11">
+        <v>0.15582008990903373</v>
+      </c>
+      <c r="K12" s="8">
         <f>IF($B$1=Tabelle2!$A$1,(1+Tabelle1!K$2)^Tabelle1!$A12,IF($B$1=Tabelle2!$A$2,(1+Tabelle1!K$2)^(-Tabelle1!$A12),IF($B$1=Tabelle2!$A$3,((1+Tabelle1!K$2)^Tabelle1!$A12-1)/(Tabelle1!K$2*(1+Tabelle1!K$2)^Tabelle1!$A12),IF($B$1=Tabelle2!$A$4,(Tabelle1!K$2*(1+Tabelle1!K$2)^Tabelle1!$A12)/((1+Tabelle1!K$2)^Tabelle1!$A12-1)))))</f>
-        <v>6.1445671057046853</v>
-      </c>
-      <c r="L12" s="11">
+        <v>0.16274539488251155</v>
+      </c>
+      <c r="L12" s="8">
         <f>IF($B$1=Tabelle2!$A$1,(1+Tabelle1!L$2)^Tabelle1!$A12,IF($B$1=Tabelle2!$A$2,(1+Tabelle1!L$2)^(-Tabelle1!$A12),IF($B$1=Tabelle2!$A$3,((1+Tabelle1!L$2)^Tabelle1!$A12-1)/(Tabelle1!L$2*(1+Tabelle1!L$2)^Tabelle1!$A12),IF($B$1=Tabelle2!$A$4,(Tabelle1!L$2*(1+Tabelle1!L$2)^Tabelle1!$A12)/((1+Tabelle1!L$2)^Tabelle1!$A12-1)))))</f>
-        <v>5.8892320111412104</v>
-      </c>
-      <c r="M12" s="11">
+        <v>0.16980142709749024</v>
+      </c>
+      <c r="M12" s="8">
         <f>IF($B$1=Tabelle2!$A$1,(1+Tabelle1!M$2)^Tabelle1!$A12,IF($B$1=Tabelle2!$A$2,(1+Tabelle1!M$2)^(-Tabelle1!$A12),IF($B$1=Tabelle2!$A$3,((1+Tabelle1!M$2)^Tabelle1!$A12-1)/(Tabelle1!M$2*(1+Tabelle1!M$2)^Tabelle1!$A12),IF($B$1=Tabelle2!$A$4,(Tabelle1!M$2*(1+Tabelle1!M$2)^Tabelle1!$A12)/((1+Tabelle1!M$2)^Tabelle1!$A12-1)))))</f>
-        <v>5.6502230284108661</v>
+        <v>0.17698416415984405</v>
       </c>
     </row>
     <row r="13" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A13" s="6">
         <v>15</v>
       </c>
-      <c r="B13" s="11">
+      <c r="B13" s="8">
         <f>IF($B$1=Tabelle2!$A$1,(1+Tabelle1!B$2)^Tabelle1!$A13,IF($B$1=Tabelle2!$A$2,(1+Tabelle1!B$2)^(-Tabelle1!$A13),IF($B$1=Tabelle2!$A$3,((1+Tabelle1!B$2)^Tabelle1!$A13-1)/(Tabelle1!B$2*(1+Tabelle1!B$2)^Tabelle1!$A13),IF($B$1=Tabelle2!$A$4,(Tabelle1!B$2*(1+Tabelle1!B$2)^Tabelle1!$A13)/((1+Tabelle1!B$2)^Tabelle1!$A13-1)))))</f>
-        <v>13.865052517162095</v>
-      </c>
-      <c r="C13" s="11">
+        <v>7.2123780184907699E-2</v>
+      </c>
+      <c r="C13" s="8">
         <f>IF($B$1=Tabelle2!$A$1,(1+Tabelle1!C$2)^Tabelle1!$A13,IF($B$1=Tabelle2!$A$2,(1+Tabelle1!C$2)^(-Tabelle1!$A13),IF($B$1=Tabelle2!$A$3,((1+Tabelle1!C$2)^Tabelle1!$A13-1)/(Tabelle1!C$2*(1+Tabelle1!C$2)^Tabelle1!$A13),IF($B$1=Tabelle2!$A$4,(Tabelle1!C$2*(1+Tabelle1!C$2)^Tabelle1!$A13)/((1+Tabelle1!C$2)^Tabelle1!$A13-1)))))</f>
-        <v>12.849263500574036</v>
-      </c>
-      <c r="D13" s="11">
+        <v>7.7825472250244179E-2</v>
+      </c>
+      <c r="D13" s="8">
         <f>IF($B$1=Tabelle2!$A$1,(1+Tabelle1!D$2)^Tabelle1!$A13,IF($B$1=Tabelle2!$A$2,(1+Tabelle1!D$2)^(-Tabelle1!$A13),IF($B$1=Tabelle2!$A$3,((1+Tabelle1!D$2)^Tabelle1!$A13-1)/(Tabelle1!D$2*(1+Tabelle1!D$2)^Tabelle1!$A13),IF($B$1=Tabelle2!$A$4,(Tabelle1!D$2*(1+Tabelle1!D$2)^Tabelle1!$A13)/((1+Tabelle1!D$2)^Tabelle1!$A13-1)))))</f>
-        <v>11.937935086776077</v>
-      </c>
-      <c r="E13" s="11">
+        <v>8.3766580462288048E-2</v>
+      </c>
+      <c r="E13" s="8">
         <f>IF($B$1=Tabelle2!$A$1,(1+Tabelle1!E$2)^Tabelle1!$A13,IF($B$1=Tabelle2!$A$2,(1+Tabelle1!E$2)^(-Tabelle1!$A13),IF($B$1=Tabelle2!$A$3,((1+Tabelle1!E$2)^Tabelle1!$A13-1)/(Tabelle1!E$2*(1+Tabelle1!E$2)^Tabelle1!$A13),IF($B$1=Tabelle2!$A$4,(Tabelle1!E$2*(1+Tabelle1!E$2)^Tabelle1!$A13)/((1+Tabelle1!E$2)^Tabelle1!$A13-1)))))</f>
-        <v>11.118387432168129</v>
-      </c>
-      <c r="F13" s="11">
+        <v>8.9941100370973137E-2</v>
+      </c>
+      <c r="F13" s="8">
         <f>IF($B$1=Tabelle2!$A$1,(1+Tabelle1!F$2)^Tabelle1!$A13,IF($B$1=Tabelle2!$A$2,(1+Tabelle1!F$2)^(-Tabelle1!$A13),IF($B$1=Tabelle2!$A$3,((1+Tabelle1!F$2)^Tabelle1!$A13-1)/(Tabelle1!F$2*(1+Tabelle1!F$2)^Tabelle1!$A13),IF($B$1=Tabelle2!$A$4,(Tabelle1!F$2*(1+Tabelle1!F$2)^Tabelle1!$A13)/((1+Tabelle1!F$2)^Tabelle1!$A13-1)))))</f>
-        <v>10.379658038180596</v>
-      </c>
-      <c r="G13" s="11">
+        <v>9.6342287609244348E-2</v>
+      </c>
+      <c r="G13" s="8">
         <f>IF($B$1=Tabelle2!$A$1,(1+Tabelle1!G$2)^Tabelle1!$A13,IF($B$1=Tabelle2!$A$2,(1+Tabelle1!G$2)^(-Tabelle1!$A13),IF($B$1=Tabelle2!$A$3,((1+Tabelle1!G$2)^Tabelle1!$A13-1)/(Tabelle1!G$2*(1+Tabelle1!G$2)^Tabelle1!$A13),IF($B$1=Tabelle2!$A$4,(Tabelle1!G$2*(1+Tabelle1!G$2)^Tabelle1!$A13)/((1+Tabelle1!G$2)^Tabelle1!$A13-1)))))</f>
-        <v>9.7122489877409954</v>
-      </c>
-      <c r="H13" s="11">
+        <v>0.10296276395531262</v>
+      </c>
+      <c r="H13" s="8">
         <f>IF($B$1=Tabelle2!$A$1,(1+Tabelle1!H$2)^Tabelle1!$A13,IF($B$1=Tabelle2!$A$2,(1+Tabelle1!H$2)^(-Tabelle1!$A13),IF($B$1=Tabelle2!$A$3,((1+Tabelle1!H$2)^Tabelle1!$A13-1)/(Tabelle1!H$2*(1+Tabelle1!H$2)^Tabelle1!$A13),IF($B$1=Tabelle2!$A$4,(Tabelle1!H$2*(1+Tabelle1!H$2)^Tabelle1!$A13)/((1+Tabelle1!H$2)^Tabelle1!$A13-1)))))</f>
-        <v>9.1079140051091478</v>
-      </c>
-      <c r="I13" s="11">
+        <v>0.10979462470100652</v>
+      </c>
+      <c r="I13" s="8">
         <f>IF($B$1=Tabelle2!$A$1,(1+Tabelle1!I$2)^Tabelle1!$A13,IF($B$1=Tabelle2!$A$2,(1+Tabelle1!I$2)^(-Tabelle1!$A13),IF($B$1=Tabelle2!$A$3,((1+Tabelle1!I$2)^Tabelle1!$A13-1)/(Tabelle1!I$2*(1+Tabelle1!I$2)^Tabelle1!$A13),IF($B$1=Tabelle2!$A$4,(Tabelle1!I$2*(1+Tabelle1!I$2)^Tabelle1!$A13)/((1+Tabelle1!I$2)^Tabelle1!$A13-1)))))</f>
-        <v>8.5594786879263758</v>
-      </c>
-      <c r="J13" s="11">
+        <v>0.11682954493601999</v>
+      </c>
+      <c r="J13" s="8">
         <f>IF($B$1=Tabelle2!$A$1,(1+Tabelle1!J$2)^Tabelle1!$A13,IF($B$1=Tabelle2!$A$2,(1+Tabelle1!J$2)^(-Tabelle1!$A13),IF($B$1=Tabelle2!$A$3,((1+Tabelle1!J$2)^Tabelle1!$A13-1)/(Tabelle1!J$2*(1+Tabelle1!J$2)^Tabelle1!$A13),IF($B$1=Tabelle2!$A$4,(Tabelle1!J$2*(1+Tabelle1!J$2)^Tabelle1!$A13)/((1+Tabelle1!J$2)^Tabelle1!$A13-1)))))</f>
-        <v>8.0606884298542472</v>
-      </c>
-      <c r="K13" s="11">
+        <v>0.12405888265031004</v>
+      </c>
+      <c r="K13" s="8">
         <f>IF($B$1=Tabelle2!$A$1,(1+Tabelle1!K$2)^Tabelle1!$A13,IF($B$1=Tabelle2!$A$2,(1+Tabelle1!K$2)^(-Tabelle1!$A13),IF($B$1=Tabelle2!$A$3,((1+Tabelle1!K$2)^Tabelle1!$A13-1)/(Tabelle1!K$2*(1+Tabelle1!K$2)^Tabelle1!$A13),IF($B$1=Tabelle2!$A$4,(Tabelle1!K$2*(1+Tabelle1!K$2)^Tabelle1!$A13)/((1+Tabelle1!K$2)^Tabelle1!$A13-1)))))</f>
-        <v>7.6060795063083662</v>
-      </c>
-      <c r="L13" s="11">
+        <v>0.13147377688737219</v>
+      </c>
+      <c r="L13" s="8">
         <f>IF($B$1=Tabelle2!$A$1,(1+Tabelle1!L$2)^Tabelle1!$A13,IF($B$1=Tabelle2!$A$2,(1+Tabelle1!L$2)^(-Tabelle1!$A13),IF($B$1=Tabelle2!$A$3,((1+Tabelle1!L$2)^Tabelle1!$A13-1)/(Tabelle1!L$2*(1+Tabelle1!L$2)^Tabelle1!$A13),IF($B$1=Tabelle2!$A$4,(Tabelle1!L$2*(1+Tabelle1!L$2)^Tabelle1!$A13)/((1+Tabelle1!L$2)^Tabelle1!$A13-1)))))</f>
-        <v>7.1908695759061931</v>
-      </c>
-      <c r="M13" s="11">
+        <v>0.13906523952966843</v>
+      </c>
+      <c r="M13" s="8">
         <f>IF($B$1=Tabelle2!$A$1,(1+Tabelle1!M$2)^Tabelle1!$A13,IF($B$1=Tabelle2!$A$2,(1+Tabelle1!M$2)^(-Tabelle1!$A13),IF($B$1=Tabelle2!$A$3,((1+Tabelle1!M$2)^Tabelle1!$A13-1)/(Tabelle1!M$2*(1+Tabelle1!M$2)^Tabelle1!$A13),IF($B$1=Tabelle2!$A$4,(Tabelle1!M$2*(1+Tabelle1!M$2)^Tabelle1!$A13)/((1+Tabelle1!M$2)^Tabelle1!$A13-1)))))</f>
-        <v>6.8108644894650059</v>
+        <v>0.14682423964634631</v>
       </c>
     </row>
     <row r="14" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A14" s="6">
         <v>20</v>
       </c>
-      <c r="B14" s="11">
+      <c r="B14" s="8">
         <f>IF($B$1=Tabelle2!$A$1,(1+Tabelle1!B$2)^Tabelle1!$A14,IF($B$1=Tabelle2!$A$2,(1+Tabelle1!B$2)^(-Tabelle1!$A14),IF($B$1=Tabelle2!$A$3,((1+Tabelle1!B$2)^Tabelle1!$A14-1)/(Tabelle1!B$2*(1+Tabelle1!B$2)^Tabelle1!$A14),IF($B$1=Tabelle2!$A$4,(Tabelle1!B$2*(1+Tabelle1!B$2)^Tabelle1!$A14)/((1+Tabelle1!B$2)^Tabelle1!$A14-1)))))</f>
-        <v>18.045552966270456</v>
-      </c>
-      <c r="C14" s="11">
+        <v>5.5415314890551334E-2</v>
+      </c>
+      <c r="C14" s="8">
         <f>IF($B$1=Tabelle2!$A$1,(1+Tabelle1!C$2)^Tabelle1!$A14,IF($B$1=Tabelle2!$A$2,(1+Tabelle1!C$2)^(-Tabelle1!$A14),IF($B$1=Tabelle2!$A$3,((1+Tabelle1!C$2)^Tabelle1!$A14-1)/(Tabelle1!C$2*(1+Tabelle1!C$2)^Tabelle1!$A14),IF($B$1=Tabelle2!$A$4,(Tabelle1!C$2*(1+Tabelle1!C$2)^Tabelle1!$A14)/((1+Tabelle1!C$2)^Tabelle1!$A14-1)))))</f>
-        <v>16.351433344597112</v>
-      </c>
-      <c r="D14" s="11">
+        <v>6.1156718125290395E-2</v>
+      </c>
+      <c r="D14" s="8">
         <f>IF($B$1=Tabelle2!$A$1,(1+Tabelle1!D$2)^Tabelle1!$A14,IF($B$1=Tabelle2!$A$2,(1+Tabelle1!D$2)^(-Tabelle1!$A14),IF($B$1=Tabelle2!$A$3,((1+Tabelle1!D$2)^Tabelle1!$A14-1)/(Tabelle1!D$2*(1+Tabelle1!D$2)^Tabelle1!$A14),IF($B$1=Tabelle2!$A$4,(Tabelle1!D$2*(1+Tabelle1!D$2)^Tabelle1!$A14)/((1+Tabelle1!D$2)^Tabelle1!$A14-1)))))</f>
-        <v>14.877474860455502</v>
-      </c>
-      <c r="E14" s="11">
+        <v>6.7215707596859159E-2</v>
+      </c>
+      <c r="E14" s="8">
         <f>IF($B$1=Tabelle2!$A$1,(1+Tabelle1!E$2)^Tabelle1!$A14,IF($B$1=Tabelle2!$A$2,(1+Tabelle1!E$2)^(-Tabelle1!$A14),IF($B$1=Tabelle2!$A$3,((1+Tabelle1!E$2)^Tabelle1!$A14-1)/(Tabelle1!E$2*(1+Tabelle1!E$2)^Tabelle1!$A14),IF($B$1=Tabelle2!$A$4,(Tabelle1!E$2*(1+Tabelle1!E$2)^Tabelle1!$A14)/((1+Tabelle1!E$2)^Tabelle1!$A14-1)))))</f>
-        <v>13.590326344967698</v>
-      </c>
-      <c r="F14" s="11">
+        <v>7.3581750328628834E-2</v>
+      </c>
+      <c r="F14" s="8">
         <f>IF($B$1=Tabelle2!$A$1,(1+Tabelle1!F$2)^Tabelle1!$A14,IF($B$1=Tabelle2!$A$2,(1+Tabelle1!F$2)^(-Tabelle1!$A14),IF($B$1=Tabelle2!$A$3,((1+Tabelle1!F$2)^Tabelle1!$A14-1)/(Tabelle1!F$2*(1+Tabelle1!F$2)^Tabelle1!$A14),IF($B$1=Tabelle2!$A$4,(Tabelle1!F$2*(1+Tabelle1!F$2)^Tabelle1!$A14)/((1+Tabelle1!F$2)^Tabelle1!$A14-1)))))</f>
-        <v>12.462210342539986</v>
-      </c>
-      <c r="G14" s="11">
+        <v>8.0242587190691314E-2</v>
+      </c>
+      <c r="G14" s="8">
         <f>IF($B$1=Tabelle2!$A$1,(1+Tabelle1!G$2)^Tabelle1!$A14,IF($B$1=Tabelle2!$A$2,(1+Tabelle1!G$2)^(-Tabelle1!$A14),IF($B$1=Tabelle2!$A$3,((1+Tabelle1!G$2)^Tabelle1!$A14-1)/(Tabelle1!G$2*(1+Tabelle1!G$2)^Tabelle1!$A14),IF($B$1=Tabelle2!$A$4,(Tabelle1!G$2*(1+Tabelle1!G$2)^Tabelle1!$A14)/((1+Tabelle1!G$2)^Tabelle1!$A14-1)))))</f>
-        <v>11.469921218565263</v>
-      </c>
-      <c r="H14" s="11">
+        <v>8.7184556976851402E-2</v>
+      </c>
+      <c r="H14" s="8">
         <f>IF($B$1=Tabelle2!$A$1,(1+Tabelle1!H$2)^Tabelle1!$A14,IF($B$1=Tabelle2!$A$2,(1+Tabelle1!H$2)^(-Tabelle1!$A14),IF($B$1=Tabelle2!$A$3,((1+Tabelle1!H$2)^Tabelle1!$A14-1)/(Tabelle1!H$2*(1+Tabelle1!H$2)^Tabelle1!$A14),IF($B$1=Tabelle2!$A$4,(Tabelle1!H$2*(1+Tabelle1!H$2)^Tabelle1!$A14)/((1+Tabelle1!H$2)^Tabelle1!$A14-1)))))</f>
-        <v>10.59401424551616</v>
-      </c>
-      <c r="I14" s="11">
+        <v>9.4392925743255696E-2</v>
+      </c>
+      <c r="I14" s="8">
         <f>IF($B$1=Tabelle2!$A$1,(1+Tabelle1!I$2)^Tabelle1!$A14,IF($B$1=Tabelle2!$A$2,(1+Tabelle1!I$2)^(-Tabelle1!$A14),IF($B$1=Tabelle2!$A$3,((1+Tabelle1!I$2)^Tabelle1!$A14-1)/(Tabelle1!I$2*(1+Tabelle1!I$2)^Tabelle1!$A14),IF($B$1=Tabelle2!$A$4,(Tabelle1!I$2*(1+Tabelle1!I$2)^Tabelle1!$A14)/((1+Tabelle1!I$2)^Tabelle1!$A14-1)))))</f>
-        <v>9.8181474074492936</v>
-      </c>
-      <c r="J14" s="11">
+        <v>0.10185220882315059</v>
+      </c>
+      <c r="J14" s="8">
         <f>IF($B$1=Tabelle2!$A$1,(1+Tabelle1!J$2)^Tabelle1!$A14,IF($B$1=Tabelle2!$A$2,(1+Tabelle1!J$2)^(-Tabelle1!$A14),IF($B$1=Tabelle2!$A$3,((1+Tabelle1!J$2)^Tabelle1!$A14-1)/(Tabelle1!J$2*(1+Tabelle1!J$2)^Tabelle1!$A14),IF($B$1=Tabelle2!$A$4,(Tabelle1!J$2*(1+Tabelle1!J$2)^Tabelle1!$A14)/((1+Tabelle1!J$2)^Tabelle1!$A14-1)))))</f>
-        <v>9.1285456690859235</v>
-      </c>
-      <c r="K14" s="11">
+        <v>0.10954647500822921</v>
+      </c>
+      <c r="K14" s="8">
         <f>IF($B$1=Tabelle2!$A$1,(1+Tabelle1!K$2)^Tabelle1!$A14,IF($B$1=Tabelle2!$A$2,(1+Tabelle1!K$2)^(-Tabelle1!$A14),IF($B$1=Tabelle2!$A$3,((1+Tabelle1!K$2)^Tabelle1!$A14-1)/(Tabelle1!K$2*(1+Tabelle1!K$2)^Tabelle1!$A14),IF($B$1=Tabelle2!$A$4,(Tabelle1!K$2*(1+Tabelle1!K$2)^Tabelle1!$A14)/((1+Tabelle1!K$2)^Tabelle1!$A14-1)))))</f>
-        <v>8.5135637197585652</v>
-      </c>
-      <c r="L14" s="11">
+        <v>0.11745962477254576</v>
+      </c>
+      <c r="L14" s="8">
         <f>IF($B$1=Tabelle2!$A$1,(1+Tabelle1!L$2)^Tabelle1!$A14,IF($B$1=Tabelle2!$A$2,(1+Tabelle1!L$2)^(-Tabelle1!$A14),IF($B$1=Tabelle2!$A$3,((1+Tabelle1!L$2)^Tabelle1!$A14-1)/(Tabelle1!L$2*(1+Tabelle1!L$2)^Tabelle1!$A14),IF($B$1=Tabelle2!$A$4,(Tabelle1!L$2*(1+Tabelle1!L$2)^Tabelle1!$A14)/((1+Tabelle1!L$2)^Tabelle1!$A14-1)))))</f>
-        <v>7.9633281173668822</v>
-      </c>
-      <c r="M14" s="11">
+        <v>0.12557563687714221</v>
+      </c>
+      <c r="M14" s="8">
         <f>IF($B$1=Tabelle2!$A$1,(1+Tabelle1!M$2)^Tabelle1!$A14,IF($B$1=Tabelle2!$A$2,(1+Tabelle1!M$2)^(-Tabelle1!$A14),IF($B$1=Tabelle2!$A$3,((1+Tabelle1!M$2)^Tabelle1!$A14-1)/(Tabelle1!M$2*(1+Tabelle1!M$2)^Tabelle1!$A14),IF($B$1=Tabelle2!$A$4,(Tabelle1!M$2*(1+Tabelle1!M$2)^Tabelle1!$A14)/((1+Tabelle1!M$2)^Tabelle1!$A14-1)))))</f>
-        <v>7.4694436243275968</v>
+        <v>0.13387878003966064</v>
       </c>
     </row>
     <row r="15" spans="1:13" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A15" s="7">
         <v>25</v>
       </c>
-      <c r="B15" s="11">
+      <c r="B15" s="8">
         <f>IF($B$1=Tabelle2!$A$1,(1+Tabelle1!B$2)^Tabelle1!$A15,IF($B$1=Tabelle2!$A$2,(1+Tabelle1!B$2)^(-Tabelle1!$A15),IF($B$1=Tabelle2!$A$3,((1+Tabelle1!B$2)^Tabelle1!$A15-1)/(Tabelle1!B$2*(1+Tabelle1!B$2)^Tabelle1!$A15),IF($B$1=Tabelle2!$A$4,(Tabelle1!B$2*(1+Tabelle1!B$2)^Tabelle1!$A15)/((1+Tabelle1!B$2)^Tabelle1!$A15-1)))))</f>
-        <v>22.023155700621672</v>
-      </c>
-      <c r="C15" s="11">
+        <v>4.540675340054795E-2</v>
+      </c>
+      <c r="C15" s="8">
         <f>IF($B$1=Tabelle2!$A$1,(1+Tabelle1!C$2)^Tabelle1!$A15,IF($B$1=Tabelle2!$A$2,(1+Tabelle1!C$2)^(-Tabelle1!$A15),IF($B$1=Tabelle2!$A$3,((1+Tabelle1!C$2)^Tabelle1!$A15-1)/(Tabelle1!C$2*(1+Tabelle1!C$2)^Tabelle1!$A15),IF($B$1=Tabelle2!$A$4,(Tabelle1!C$2*(1+Tabelle1!C$2)^Tabelle1!$A15)/((1+Tabelle1!C$2)^Tabelle1!$A15-1)))))</f>
-        <v>19.523456473586034</v>
-      </c>
-      <c r="D15" s="11">
+        <v>5.122043841739473E-2</v>
+      </c>
+      <c r="D15" s="8">
         <f>IF($B$1=Tabelle2!$A$1,(1+Tabelle1!D$2)^Tabelle1!$A15,IF($B$1=Tabelle2!$A$2,(1+Tabelle1!D$2)^(-Tabelle1!$A15),IF($B$1=Tabelle2!$A$3,((1+Tabelle1!D$2)^Tabelle1!$A15-1)/(Tabelle1!D$2*(1+Tabelle1!D$2)^Tabelle1!$A15),IF($B$1=Tabelle2!$A$4,(Tabelle1!D$2*(1+Tabelle1!D$2)^Tabelle1!$A15)/((1+Tabelle1!D$2)^Tabelle1!$A15-1)))))</f>
-        <v>17.413147691278013</v>
-      </c>
-      <c r="E15" s="11">
+        <v>5.7427871039127817E-2</v>
+      </c>
+      <c r="E15" s="8">
         <f>IF($B$1=Tabelle2!$A$1,(1+Tabelle1!E$2)^Tabelle1!$A15,IF($B$1=Tabelle2!$A$2,(1+Tabelle1!E$2)^(-Tabelle1!$A15),IF($B$1=Tabelle2!$A$3,((1+Tabelle1!E$2)^Tabelle1!$A15-1)/(Tabelle1!E$2*(1+Tabelle1!E$2)^Tabelle1!$A15),IF($B$1=Tabelle2!$A$4,(Tabelle1!E$2*(1+Tabelle1!E$2)^Tabelle1!$A15)/((1+Tabelle1!E$2)^Tabelle1!$A15-1)))))</f>
-        <v>15.622079943650904</v>
-      </c>
-      <c r="F15" s="11">
+        <v>6.4011962786454574E-2</v>
+      </c>
+      <c r="F15" s="8">
         <f>IF($B$1=Tabelle2!$A$1,(1+Tabelle1!F$2)^Tabelle1!$A15,IF($B$1=Tabelle2!$A$2,(1+Tabelle1!F$2)^(-Tabelle1!$A15),IF($B$1=Tabelle2!$A$3,((1+Tabelle1!F$2)^Tabelle1!$A15-1)/(Tabelle1!F$2*(1+Tabelle1!F$2)^Tabelle1!$A15),IF($B$1=Tabelle2!$A$4,(Tabelle1!F$2*(1+Tabelle1!F$2)^Tabelle1!$A15)/((1+Tabelle1!F$2)^Tabelle1!$A15-1)))))</f>
-        <v>14.093944566044758</v>
-      </c>
-      <c r="G15" s="11">
+        <v>7.0952457299229624E-2</v>
+      </c>
+      <c r="G15" s="8">
         <f>IF($B$1=Tabelle2!$A$1,(1+Tabelle1!G$2)^Tabelle1!$A15,IF($B$1=Tabelle2!$A$2,(1+Tabelle1!G$2)^(-Tabelle1!$A15),IF($B$1=Tabelle2!$A$3,((1+Tabelle1!G$2)^Tabelle1!$A15-1)/(Tabelle1!G$2*(1+Tabelle1!G$2)^Tabelle1!$A15),IF($B$1=Tabelle2!$A$4,(Tabelle1!G$2*(1+Tabelle1!G$2)^Tabelle1!$A15)/((1+Tabelle1!G$2)^Tabelle1!$A15-1)))))</f>
-        <v>12.783356158268411</v>
-      </c>
-      <c r="H15" s="11">
+        <v>7.8226718212273949E-2</v>
+      </c>
+      <c r="H15" s="8">
         <f>IF($B$1=Tabelle2!$A$1,(1+Tabelle1!H$2)^Tabelle1!$A15,IF($B$1=Tabelle2!$A$2,(1+Tabelle1!H$2)^(-Tabelle1!$A15),IF($B$1=Tabelle2!$A$3,((1+Tabelle1!H$2)^Tabelle1!$A15-1)/(Tabelle1!H$2*(1+Tabelle1!H$2)^Tabelle1!$A15),IF($B$1=Tabelle2!$A$4,(Tabelle1!H$2*(1+Tabelle1!H$2)^Tabelle1!$A15)/((1+Tabelle1!H$2)^Tabelle1!$A15-1)))))</f>
-        <v>11.65358317825372</v>
-      </c>
-      <c r="I15" s="11">
+        <v>8.5810517220665614E-2</v>
+      </c>
+      <c r="I15" s="8">
         <f>IF($B$1=Tabelle2!$A$1,(1+Tabelle1!I$2)^Tabelle1!$A15,IF($B$1=Tabelle2!$A$2,(1+Tabelle1!I$2)^(-Tabelle1!$A15),IF($B$1=Tabelle2!$A$3,((1+Tabelle1!I$2)^Tabelle1!$A15-1)/(Tabelle1!I$2*(1+Tabelle1!I$2)^Tabelle1!$A15),IF($B$1=Tabelle2!$A$4,(Tabelle1!I$2*(1+Tabelle1!I$2)^Tabelle1!$A15)/((1+Tabelle1!I$2)^Tabelle1!$A15-1)))))</f>
-        <v>10.674776188588581</v>
-      </c>
-      <c r="J15" s="11">
+        <v>9.3678779051968114E-2</v>
+      </c>
+      <c r="J15" s="8">
         <f>IF($B$1=Tabelle2!$A$1,(1+Tabelle1!J$2)^Tabelle1!$A15,IF($B$1=Tabelle2!$A$2,(1+Tabelle1!J$2)^(-Tabelle1!$A15),IF($B$1=Tabelle2!$A$3,((1+Tabelle1!J$2)^Tabelle1!$A15-1)/(Tabelle1!J$2*(1+Tabelle1!J$2)^Tabelle1!$A15),IF($B$1=Tabelle2!$A$4,(Tabelle1!J$2*(1+Tabelle1!J$2)^Tabelle1!$A15)/((1+Tabelle1!J$2)^Tabelle1!$A15-1)))))</f>
-        <v>9.8225796049484888</v>
-      </c>
-      <c r="K15" s="11">
+        <v>0.10180625051857181</v>
+      </c>
+      <c r="K15" s="8">
         <f>IF($B$1=Tabelle2!$A$1,(1+Tabelle1!K$2)^Tabelle1!$A15,IF($B$1=Tabelle2!$A$2,(1+Tabelle1!K$2)^(-Tabelle1!$A15),IF($B$1=Tabelle2!$A$3,((1+Tabelle1!K$2)^Tabelle1!$A15-1)/(Tabelle1!K$2*(1+Tabelle1!K$2)^Tabelle1!$A15),IF($B$1=Tabelle2!$A$4,(Tabelle1!K$2*(1+Tabelle1!K$2)^Tabelle1!$A15)/((1+Tabelle1!K$2)^Tabelle1!$A15-1)))))</f>
-        <v>9.0770400182293596</v>
-      </c>
-      <c r="L15" s="11">
+        <v>0.11016807219002084</v>
+      </c>
+      <c r="L15" s="8">
         <f>IF($B$1=Tabelle2!$A$1,(1+Tabelle1!L$2)^Tabelle1!$A15,IF($B$1=Tabelle2!$A$2,(1+Tabelle1!L$2)^(-Tabelle1!$A15),IF($B$1=Tabelle2!$A$3,((1+Tabelle1!L$2)^Tabelle1!$A15-1)/(Tabelle1!L$2*(1+Tabelle1!L$2)^Tabelle1!$A15),IF($B$1=Tabelle2!$A$4,(Tabelle1!L$2*(1+Tabelle1!L$2)^Tabelle1!$A15)/((1+Tabelle1!L$2)^Tabelle1!$A15-1)))))</f>
-        <v>8.421744664666905</v>
-      </c>
-      <c r="M15" s="11">
+        <v>0.11874024205405564</v>
+      </c>
+      <c r="M15" s="8">
         <f>IF($B$1=Tabelle2!$A$1,(1+Tabelle1!M$2)^Tabelle1!$A15,IF($B$1=Tabelle2!$A$2,(1+Tabelle1!M$2)^(-Tabelle1!$A15),IF($B$1=Tabelle2!$A$3,((1+Tabelle1!M$2)^Tabelle1!$A15-1)/(Tabelle1!M$2*(1+Tabelle1!M$2)^Tabelle1!$A15),IF($B$1=Tabelle2!$A$4,(Tabelle1!M$2*(1+Tabelle1!M$2)^Tabelle1!$A15)/((1+Tabelle1!M$2)^Tabelle1!$A15-1)))))</f>
-        <v>7.8431391120645539</v>
+        <v>0.12749996980950773</v>
       </c>
     </row>
     <row r="17" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A17" s="14" t="str">
+      <c r="A17" s="11" t="str">
         <f>VLOOKUP($B$1,Tabelle2!$A$1:$B$4,2,FALSE)</f>
-        <v>Welchen Gegenwarts- oder Barwert hat eine n Jahre lang (nachschüssig) gezahlte gleichbleibende jährliche Rente von 1 GE?</v>
-      </c>
-      <c r="B17" s="14"/>
-      <c r="C17" s="14"/>
-      <c r="D17" s="14"/>
-      <c r="E17" s="14"/>
-      <c r="F17" s="14"/>
-      <c r="G17" s="14"/>
-      <c r="H17" s="14"/>
-      <c r="I17" s="14"/>
-      <c r="J17" s="14"/>
-      <c r="K17" s="14"/>
-      <c r="L17" s="14"/>
-      <c r="M17" s="14"/>
+        <v>Wie hoch ist die jährliche Rente, die n Jahre lang (nachschüssig) aus einem Gegenwarts- oder Barwert von 1 GE gezahlt werden kann?</v>
+      </c>
+      <c r="B17" s="11"/>
+      <c r="C17" s="11"/>
+      <c r="D17" s="11"/>
+      <c r="E17" s="11"/>
+      <c r="F17" s="11"/>
+      <c r="G17" s="11"/>
+      <c r="H17" s="11"/>
+      <c r="I17" s="11"/>
+      <c r="J17" s="11"/>
+      <c r="K17" s="11"/>
+      <c r="L17" s="11"/>
+      <c r="M17" s="11"/>
+    </row>
+    <row r="19" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="B19" s="15"/>
     </row>
   </sheetData>
   <mergeCells count="2">

</xml_diff>